<commit_message>
Add THEFT-011 to THEFT-020 to Theft Case Database — Batch 2 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Theft_Case_Database.xlsx
+++ b/knowledge/case-databases/Theft_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1653,6 +1653,1056 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="120" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>DRN2801347</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — car stolen; Aviva cancelled policy for non-disclosure of prior claims and convictions (would have offered cover on different terms so policy remained in force); spare key left in glove box by named driver Mr Y; Aviva declined theft claim under 'keys in car' policy exclusion; dispute about whether the exclusion was sufficiently highlighted in the policy summary</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft using key left in vehicle — spare key left in glove box by named driver Mr Y; vehicle stolen using that key; specific method of gain beyond key availability not described</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Spare key left in glove box of car by named driver Mr Y triggered the 'keys in car' policy exclusion; Aviva also cancelled (not voided) policy for non-disclosure — as it would have offered cover on different terms, cover was in force at time of theft but claim declined solely on the keys-in-car exclusion</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Mr T and Mr Y: 'keys in car' exclusion not sufficiently highlighted — adjudicator agreed it was 'buried' in a block of text in the policy summary. Aviva: exclusion contained in policy summary under the heading 'significant or unusual exclusions' as per FOS guidance; provided evidence it had informed Mr T the claim was declined on this exclusion. FOS (ombudsman): adjudicator found exclusion buried — ombudsman disagreed; policy summary longer than usual but first page was a cover sheet, second page very clear and easy to read, significant and unusual exclusions on third page under a bold heading; reasonable to expect Mr T to read first two or three pages of a Key Facts summary and note a bold heading for significant or unusual exclusions; exclusion sufficiently highlighted; parties made no further comment after provisional decision.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Aviva acted fairly and reasonably in declining the theft claim; 'keys in car' exclusion was sufficiently highlighted in the policy summary</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>'Keys in car' exclusion is enforceable where placed under a bold 'significant or unusual exclusions' heading in a Key Facts policy summary — even on page 3 of a longer-than-usual summary; consumer is expected to read at least the first two or three pages of a Key Facts summary and note a distinct bold heading for significant or unusual exclusions; where an insurer cancels (rather than voids) for non-disclosure because it would have offered cover on different terms, the policy remains in force at the time of the claim and exclusions still apply; a spare key left in the vehicle by a named driver triggers the keys-in-car exclusion regardless of whether the policyholder was aware the key was there</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>Specific details of why Mr Y left the spare key in the glove box and whether Mr T was aware of its presence</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>Adjudicator concluded exclusion was 'buried' in a block of text on page 3 of the policy summary; ombudsman reviewed summary — first page is a cover sheet, second page very clear and easy to read, significant and unusual exclusions on page 3 under a bold heading; not unreasonable to expect policyholder to read first two or three pages of a Key Facts summary; bold heading makes exclusion locatable; exclusion was sufficiently highlighted; Aviva correctly communicated decline reason to Mr T; neither party made further comment after provisional decision; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>A 'keys in car' exclusion placed under a bold 'significant or unusual exclusions' heading in the Key Facts policy summary is enforceable — even if located on page 3 of a longer-than-usual summary; when cancelling (not voiding) for non-disclosure, the policy remains in force and all exclusions continue to apply to any claim arising during the policy period; a named driver who leaves a spare key in the vehicle triggers the keys-in-car exclusion even if the main policyholder was unaware the key was there</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>IF spare_key_left_in_vehicle AND policy_contains_keys_in_car_exclusion THEN exclusion_applies_regardless_of_who_left_key; IF exclusion_listed_under_bold_significant_or_unusual_exclusions_heading_in_key_facts_summary THEN exclusion_is_sufficiently_highlighted; IF non_disclosure_leads_to_cancellation_not_voidance THEN policy_remains_in_force_and_all_exclusions_continue_to_apply</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>DRN2801347.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-012</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>DRN2886197</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Travel insurance — bag stolen from car footwell at service station during a toilet break; Mr and Mrs T took turns so one was always within 8-10 feet of the car; UKI declined as valuables and personal belongings were left 'unattended' in a motor vehicle; complainants dispute the car was ever unattended</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Theft from vehicle — bag removed from car footwell at service station while neither occupant was watching or able to notice the theft; theft entirely undetected until occupants returned to drive away; estate car meant bag could not be hidden in the boot</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Personal travel insurance</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Policy excluded cover for theft of personal possessions and valuables left in an unattended motor vehicle; UKI concluded the car was 'unattended' as neither Mr nor Mrs T was in a position to prevent the theft or even notice when someone approached</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Mr and Mrs T: car not left unattended — took turns for toilet break; one always within 8-10 feet; travelling with a dog; estate car meant bag could not be locked in boot as items visible through rear and side windows; close proximity made taking the bag unnecessary. UKI: belongings left unattended in motor vehicle — exclusion applies. FOS: accepted they took turns and one always in vicinity; but neither had any idea someone had opened the car door until about to drive away — they were not in a position to prevent or even notice the theft; car was therefore 'unattended'; distinguished from case where consumer sees theft but cannot prevent it (e.g. thief runs quickly) — those should be covered; here there was no awareness at all.</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited entitled to reject Mr and Mrs T's claim; no award made against UK Insurance Limited</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Where a travel policy excludes theft from 'unattended' motor vehicles and provides no definition, the word is given its ordinary common sense meaning — a vehicle is unattended when the owner is not in a position to prevent a theft or even to notice when someone approaches; physical proximity alone is insufficient if the owner is entirely unaware the theft is occurring; key distinction: an insurer should pay where the consumer witnesses the theft but cannot prevent it (e.g. thief runs quickly) — that is different from being wholly unaware the theft occurred</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>None material — the factual circumstances were accepted by both parties; the dispute turned entirely on the legal interpretation of 'unattended'</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>Policy excludes theft from 'unattended' motor vehicle; no policy definition so ordinary common sense meaning applies; accepted Mr and Mrs T took turns and one always in vicinity with dog; but both letters confirm neither had any inkling someone had opened the car door until about to drive away — they were not 'attending' to the car or possessions inside it; key distinction: if consumer witnesses theft and fails to prevent it (e.g. quick thief) insurer should meet claim; here neither was aware theft was occurring — car was unattended; no reasonable basis to require UKI to make any payment</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>Travel insurance 'unattended vehicle' exclusions apply where the owner was entirely unaware the theft was occurring — physical proximity is insufficient if the owner could not notice or prevent the theft; the determinative question is whether the owner was in a position to notice and prevent the theft, not how far away they were; a consumer unable to secure valuables in a boot due to vehicle type should take the valuables with them or remain in a position to observe the vehicle interior</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>IF consumer_unaware_theft_occurred_until_after_the_fact THEN vehicle_was_unattended_for_exclusion_purposes; IF consumer_witnesses_theft_but_cannot_prevent_it THEN unattended_exclusion_does_not_apply_and_insurer_should_meet_claim; proximity_alone_insufficient_to_satisfy_attended_requirement_if_consumer_could_not_notice_or_prevent_theft</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>DRN2886197.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3028208</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Covea Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>11 Nov 2021</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — car stolen; Covea avoided (voided) policy from inception under CIDRA for non-disclosure of two 2019 speeding convictions at renewal; insured had declared one 2016 conviction; secondary complaint about £4,000 damage to recovered car alleged to have been caused by Covea's collection and storage</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft — car stolen; specific method of entry not described; key issue is non-disclosure of motoring convictions at renewal leading to policy avoidance from inception</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Mr O failed to disclose two 2019 speeding convictions at renewal — on the renewal call he said 'nothing's changed' and did not query the statement of fact which listed only the 2016 conviction; Covea's underwriting criteria (reviewed by FOS in confidence) showed it would not have offered any insurance if the two 2019 convictions had been declared; CIDRA careless qualifying misrepresentation — policy avoided from inception; premiums refunded; post-recovery damage assessed by senior engineer as consistent with theft and described as 'no or minimal' in a photo-based inspection</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Mr O: told broker about convictions at outset. Covea: renewal call recording shows Mr O said 'nothing's changed' when asked if anything had changed; statement of fact sent for checking listed only the 2016 conviction but Mr O did not query the omission; underwriting criteria (shown to FOS — confidential) demonstrates no cover would have been offered with those convictions; senior engineer confirmed reported damage is consistent with theft not with Covea's collection or storage. FOS: listened to renewal call — Mr O said 'nothing's changed' despite two new speeding convictions; had previously declared 2016 conviction so knew disclosure was required; should have noticed omission on statement of fact sent for checking; CIDRA careless qualifying misrepresentation established; avoidance + premium refund is correct remedy; post-recovery damage explanation accepted.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Covea acted fairly in avoiding motor policy from inception for careless misrepresentation under CIDRA; Covea is not responsible for post-recovery damage to Mr O's car</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Under CIDRA, answering 'nothing's changed' at renewal when two new motoring convictions exist is a careless misrepresentation — prior disclosure of one earlier conviction demonstrates the consumer knew declarations were required; the statement of fact sent for checking creates an independent obligation to verify accuracy — failure to notice the omission of material information removes any defence; insurer must evidence underwriting criteria to justify avoidance — confidential underwriting guide shown to FOS satisfies this; CIDRA remedy for careless qualifying misrepresentation where insurer would not have offered cover at all: avoid from inception and refund premiums; a photo-based post-theft vehicle inspection calibrated for total-loss assessment does not catalogue all damage — 'no or minimal damage' in that context is not equivalent to 'no damage'</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>What Mr O said to broker at original policy inception (not available); whether the broker failed to pass on any disclosure would have changed the analysis; full details of the 2019 speeding conviction dates and types (established by Covea's driving licence check during the claim call)</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>Renewal call listened to — Mr O said 'nothing's changed' despite two 2019 speeding convictions; had previously declared 2016 conviction so was aware of the disclosure obligation; statement of fact sent for checking listed only the 2016 conviction — Mr O did not query the omission; Covea underwriting criteria reviewed in confidence — no cover would have been offered with those convictions; CIDRA careless qualifying misrepresentation established; avoidance + premium refund is correct CIDRA remedy; post-recovery damage: report said 'no or minimal' (not 'no damage') and senior engineer explained £4,000 is minimal vs a £27,000 car in theft context; most damage interior and not visible in photos; report was photo-based and produced for total-loss assessment; Covea not responsible for post-collection damage</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Renewal calls with a generic 'has anything changed?' question require policyholders to proactively volunteer new convictions — answering 'no' without considering specific material changes is careless misrepresentation; the statement of fact sent for checking creates an independent verification duty — policyholders who fail to check it lose the ability to argue information was correctly provided; insurers investigating post-theft vehicle damage should clearly contextualise photo-based inspection reports (calibrated for total-loss assessment) to avoid disputes about whether 'no or minimal damage' means the vehicle sustained no damage at all</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>IF consumer_answers_nothing_changed_at_renewal AND new_convictions_exist THEN careless_misrepresentation_established; IF statement_of_fact_omits_material_information AND consumer_fails_to_notice_and_query THEN consumer_has_not_taken_reasonable_care; IF CIDRA_careless_misrepresentation AND insurer_would_not_have_offered_cover_at_all THEN avoidance_from_inception_and_premium_refund_is_correct_remedy; IF senior_engineer_confirms_damage_consistent_with_theft AND repair_cost_small_relative_to_vehicle_value THEN insurer_not_responsible_for_post_collection_damage</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3028208.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-014</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>DRN3072290</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>20 Feb 2015</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — AXA applied additional premium after discovering via the CUE database an undisclosed theft claim Mr V had made on a prior policy for a different vehicle; Mr V disputes that a claim on a separate vehicle or policy need be disclosed and argues his No Claims Discount on the current vehicle is unaffected</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Prior motor vehicle theft claim — circumstances of the prior theft on a different vehicle are not described in this decision; no current theft claim; dispute concerns whether the prior claim must be disclosed and whether AXA can apply additional premium as a result</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — current policy accepted and in force; dispute concerns AXA's entitlement to apply additional premium after discovering via CUE that Mr V had not disclosed a prior theft claim on a separate vehicle policy</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Mr V: prior claim was on a separate policy for a different vehicle; NCD earned on current vehicle and is unaffected; he has already been penalised by the previous insurer; prior claim is irrelevant to current policy. AXA: claims history transcends individual vehicles and policies; the application question asked about any motor claims in the past five years; NCD and claims history are separate considerations; additional premium was automatically calculated and is correct; AXA entitled to exercise commercial discretion in its underwriting. FOS: AXA entitled to set its own questions and premium calculation methodology; question was clear — any motor claims in past five years; prior theft claim on a separate vehicle falls within that question; NCD (vehicle-specific) and overall claims history (person-specific) are distinct; AXA legitimately exercised its commercial judgement.</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — AXA legitimately applied additional premium reflecting correct claims history; AXA was entitled to exercise its commercial judgement in its underwriting</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>A motor insurer is entitled to ask about all motor claims made in the past five years across any vehicle or policy — claims history is not vehicle-specific; No Claims Discount earned on a specific vehicle and overall claims history are separate underwriting factors that may be assessed independently; where a question about claims history is clear and comprehensive, the insurer is entitled to apply its underwriting criteria (including premium adjustments) when it discovers an undisclosed prior claim; the insurer has commercial discretion to decide which factors it uses in risk assessment and premium calculation; prior penalisation by another insurer for the same claim does not prevent a subsequent insurer from also taking that claim into account</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — factual circumstances not in dispute; the entire dispute concerned the insurer's legal entitlement to use the prior claims history in its underwriting of the current policy</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>AXA entitled to decide what questions to ask and how to calculate premiums; question was clear — any motor claims in past five years; prior theft claim on a different vehicle under a different policy falls within that question; once aware of the undisclosed claim, AXA was entitled to apply its underwriting criteria; NCD (vehicle-specific) is distinct from overall claims history (person-specific); additional premium was legitimately calculated; Mr V free to seek lower premiums from other providers if he considered AXA's premium too high</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>Policyholders must understand that prior motor claims history for insurance purposes covers all vehicles and policies — a prior theft claim on a different vehicle must be disclosed when asked about any motor claims in the past five years; NCD earned on a specific vehicle does not neutralise the insurer's right to underwrite against the policyholder's overall claims history; being previously penalised by one insurer for a claim does not prevent a subsequent insurer from independently taking that same claim into account in its risk assessment</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_asks_about_any_motor_claims_in_past_five_years THEN prior_theft_claim_on_any_vehicle_any_policy_must_be_disclosed; insurer_may_treat_NCD_and_overall_claims_history_as_separate_underwriting_factors; IF insurer_discovers_undisclosed_prior_claim_via_CUE THEN entitled_to_apply_underwriting_criteria_including_premium_adjustment; prior_penalisation_by_previous_insurer_does_not_preclude_current_insurer_from_underwriting_same_claim</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>DRN3072290.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>DRN3099586</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>22 Apr 2016</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Commercial shop and restaurant insurance — prior FOS decision required AXA to reinstate policy and settle theft and arson claims; when AXA settled the claims it paid no interest; V complains AXA should pay interest on the delayed payment and compensation for the delay</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Commercial premises theft and arson (shop/restaurant) — specific method of entry not described; this decision concerns interest on delayed claim settlement only, not the theft or arson circumstances</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Commercial (shop and restaurant insurance policy — not home/contents)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — claims accepted and settled pursuant to prior FOS decision; dispute concerns whether interest must be paid on the time-lag between the date of loss and settlement</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>V: AXA should pay interest on delayed settlement and compensation for the delay. AXA: not responsible for any avoidable delay so no interest or compensation owed. Adjudicator: interest should be paid but no compensation. AXA disagreed and requested ombudsman review. FOS (ombudsman): AXA misunderstands the purpose of interest — it is a component of indemnity to put the policyholder back in the position they would have been in if the insured event had never happened; time-lag between loss and payment requires interest regardless of whether the delay was avoidable or the insurer's fault; compensation for distress/inconvenience is distinct and only payable where avoidable delay or insurer mistakes caused additional harm — no avoidable delay here; 8% simple per annum is the appropriate interest rate.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc to pay interest (less tax if properly deductible) at 8% simple per annum on the theft claim and material damage elements of the arson claim from the respective dates of loss to the date of payment; no compensation for delay awarded</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>The principle of indemnity requires an insurer to put the policyholder back in the same position as if the insured event had not occurred — where there is a time-lag between the insured event and payment, interest must be paid to achieve true indemnity regardless of whether the delay was avoidable or the insurer's fault; interest and compensation for distress/inconvenience are distinct obligations — interest is a component of indemnity; compensation for distress is only payable where avoidable delay or insurer mistakes caused additional harm to the policyholder; FOS applies 8% simple per annum as standard interest rate on insurance settlement payments</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Precise dates of each loss event and corresponding settlement payment dates (needed to calculate interest quantum; these were not disputed in this decision)</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>Prior FOS decision required AXA to reinstate policy and settle claims; AXA settled but paid no interest; AXA argued no interest was owed because the delay was not its fault — ombudsman explains this misunderstands the purpose of interest; the indemnity principle requires interest for the time-lag between loss and payment regardless of fault; compensation for distress is separate and only arises from avoidable insurer delay or mistakes — this case required detailed investigation and AXA was not responsible for avoidable delay; no compensation; 8% simple per annum is appropriate interest rate</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>Insurers settling claims (including pursuant to FOS decisions) must include interest from the date of loss to the date of payment to achieve full indemnity — the absence of fault for the delay does not remove the interest obligation; interest should be offered proactively as part of any settlement rather than waiting to be directed; compensation for distress is a separate, additional obligation that only arises when the insurer's own avoidable fault or mistakes caused identifiable additional harm</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>IF time_lag_exists_between_date_of_loss_and_settlement_payment THEN interest_at_8_percent_simple_per_annum_is_payable_regardless_of_fault; interest_and_distress_compensation_are_distinct_obligations_and_must_not_be_conflated; IF no_avoidable_delay_or_insurer_mistakes THEN no_distress_compensation_owed_even_where_interest_is_payable; interest_must_be_included_in_any_insurance_settlement_to_achieve_the_indemnity_principle</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>DRN3099586.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>DRN3125088</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Tesco Underwriting Limited</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>6 Dec 2019</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — house burgled in December 2018; both house and car keys stolen; partner's car stolen immediately but Miss W's car was not; Tesco arranged locksmith and advised Miss W to safeguard her car; three days later Miss W's car stolen from outside home by person who had possession of the stolen key; Tesco rejected theft claim for failure to take reasonable protective steps</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft using stolen keys — house burgled; car and house keys stolen; partner's car stolen at the time of the burglary; Miss W's car not immediately taken; three days later, person holding the stolen key drove away Miss W's car from outside home; no forced entry to vehicle required as thief possessed the key</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Tesco rejected the theft claim on the grounds that Miss W failed to take reasonable steps to protect her car after being advised to do so; thief had Miss W's car key and knew where the car was kept; Miss W had access to the spare car key (she was using it) and could have moved the car to a safe location or added additional physical locks; placing bins in front of a car behind a low wall is insufficient when the thief possesses the key and knows the car's location</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Miss W and Mr J: car kept behind a wall with bins in front — reasonable protective measures; Tesco should have provided specific advice about protective measures before rejecting rather than giving examples afterwards. Tesco: Miss W was advised to safeguard her car when keys were reported stolen; spare key available — she could have moved car or added extra locks; bins behind a low wall are inadequate; apologised for failing to call back as promised and gave agent feedback. FOS: reasonable to expect Miss W to take protective steps knowing the thief had her key and knew her car's location; spare key available — she was using it; could have moved car or added locks; wall is low so car clearly visible; bins in front inadequate against a thief with a key; Tesco's failure to call back was poor service but apology + agent feedback was sufficient remedy; the short callback delay did not affect the claim outcome.</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Tesco's rejection of the theft claim was fair and reasonable; apology and agent feedback was sufficient remedy for the service failure in not calling back as promised</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Where a policyholder is aware that a thief has possession of the car key and knows the vehicle's location, a reasonable care obligation arises to take proactive protective steps before a locksmith can attend — this may include relocating the vehicle or adding physical locks; placing objects in front of a vehicle behind a low wall is not a reasonable protective measure when the thief holds the key; access to a spare key means the policyholder is in a position to move the vehicle and is expected to do so; a short unexplained delay by an insurer in calling back does not affect the claim outcome where the claim was promptly decided within three working days</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>Specific content of the advice Tesco gave Miss W when it told her to 'safeguard' her car at the time keys were reported stolen (ombudsman found general advice to safeguard was sufficient — Tesco was not required to itemise specific measures in advance)</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Miss W and Mr J knew thief had key and knew car location — obligation to take reasonable protective steps arose at that point; spare key available — Miss W was using it; could have moved car to safe location or added extra locks; photo shows car visible over low wall; bins in front of car inadequate against a thief who holds the key; Tesco's failure to call back acknowledged — apology and agent feedback is sufficient remedy; three-working-day delay in calling back did not affect outcome as claim was then promptly decided; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>A theft claim may be declined where the policyholder was forewarned that the thief had the car key and knew the vehicle location, but failed to take available protective steps (such as relocating the vehicle) before a locksmith attended; the availability of a spare key is a critical factor — if the policyholder can access the vehicle they are expected to take protective action; an insurer's service failure in not making a promised callback does not affect the claim outcome if the claim was handled and decided promptly overall</t>
+        </is>
+      </c>
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>IF policyholder_aware_thief_holds_car_key AND knows_vehicle_location AND spare_key_available THEN policyholder_must_take_reasonable_protective_steps_including_relocating_vehicle; IF protective_measures_inadequate_against_keyed_access THEN reasonable_care_obligation_not_met_and_claim_may_be_declined; IF insurer_service_failure_did_not_affect_claim_outcome THEN apology_and_internal_feedback_is_proportionate_remedy</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>DRN3125088.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3197736</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>AmTrust Europe Limited</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>19 Jan 2022</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Gadget insurance — laptop noticed missing at airport during check-in for return flight from overseas trip; AmTrust declined for two reasons: (1) laptop stored in cargo hold — later conceded this was a misunderstanding of Mr A's account; (2) travelling against FCO advice — policy general exclusion 33 requires the claim to be 'a direct result' of such travel; FOS found that health-related FCO advice is not causally linked to a theft and the 'direct result' test was not met</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Theft at airport — laptop noticed missing at airport check-in for return flight; Mr A reported to airport security but left family to follow up as he needed to catch his flight; exact method of theft not established; Mr A believed it was stolen not lost</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Personal gadget insurance (laptop — standalone gadget policy, not home/contents)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>(1) Laptop stored in cargo hold — exclusion for hold storage applied; AmTrust later conceded this was a misunderstanding of Mr A's account. (2) Mr A had travelled against FCO advice — policy general exclusion 33 excludes claims that occur 'as a direct result' of travelling to a country where the FCO advise against all (but essential) travel</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Mr A: laptop was not in cargo hold; had valid personal reasons for travel; FCO advice was health-related and has no causal link to a theft. AmTrust: cargo hold exclusion applied (later conceded incorrect); FCO exclusion 33 still applies as Mr A travelled against FCO advice. FOS: cargo hold misunderstanding resolved during call and confirmed in AmTrust's FOS response; FCO advice was health-related — a health advisory does not carry a close causal relationship to the theft of a laptop; the word 'direct' in 'direct result' requires a close causal connection between the nature of the FCO advice and the specific loss; the risk of laptop theft was not heightened by a health advisory; exclusion 33 cannot fairly be applied.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>AmTrust Europe Limited must reconsider Mr A's theft claim under his policy in line with the remaining terms and conditions, without relying on general exclusion 33 (travelling against FCO advice); FOS is not directing AmTrust to pay the claim — it may still assess the claim on remaining policy terms</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>An FCO travel exclusion requiring a claim to be 'a direct result' of travelling against advice demands a close causal connection between the nature of the FCO advice and the specific type of loss claimed — 'direct' means more than temporal or geographic coincidence; where FCO advice is health-related, it does not carry a direct causal relationship to a theft loss — health advice does not increase the risk of theft; an insurer cannot rely on an FCO exclusion unless the particular advisory directly caused or heightened the risk of the specific type of loss sustained; where an insurer declines on an incorrect factual premise (cargo hold) that is later conceded, remaining grounds are examined carefully</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Valid police crime reference report from local authorities (required by policy definition of theft — Mr A reported to airport security and left family to follow up; whether a valid crime reference was ever obtained is unclear and remains for AmTrust to assess on reconsideration)</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>Cargo hold misunderstanding resolved — AmTrust confirmed in the call and in its FOS response; FCO exclusion 33 requires claim to be a 'direct result' of FCO travel advice; 'direct' denotes a close causal connection — not merely 'as a result'; FCO advice was health-related; a health advisory has no close causal link to the theft of a laptop; the risk of theft was not heightened by the health-related FCO advice; exclusion 33 cannot fairly be applied; AmTrust must reconsider without relying on that exclusion; FOS is not directing payment — AmTrust may assess the claim on remaining policy terms</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>When relying on an FCO exclusion with a 'direct result' causation test, the insurer must assess whether the nature of the FCO advice (health, security, political unrest) is causally linked to the specific type of loss — health advisories do not increase theft risk and cannot be treated as directly causing a theft; insurers should not decline on a factual misunderstanding and then rely on an exclusion whose own causation test is not satisfied; 'direct result' exclusions require analysis of the causal chain, not just the presence of FCO advice</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>IF FCO_exclusion_requires_direct_result AND FCO_advice_is_health_related AND claim_is_for_theft THEN direct_causation_test_not_met_and_exclusion_cannot_apply; direct_result_means_close_causal_connection_between_nature_of_FCO_advice_and_specific_type_of_loss; IF insurer_declines_on_factual_misunderstanding_later_conceded AND remaining_exclusion_fails_causation_test THEN claim_must_be_reconsidered_on_remaining_policy_terms</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3197736.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-018</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>DRN3351038</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Liverpool Victoria Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>25 Apr 2016</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Household contents insurance — 2015 home burglary; more than £20,000 of jewellery stolen; LV applied a valuables limit of £5,000 and paid a further £3,000 for unspecified personal possessions; Mr G claims LV told him at inception (2002) that these limits would not apply to theft claims</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Burglary — home broken into in 2015; more than £20,000 of jewellery stolen; specific method of forced entry not described in the decision</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — theft claim accepted but settled at the policy's valuables limit (£5,000) and unspecified personal possessions sub-limit (£3,000); Mr G disputes the application of these limits, claiming they do not apply to theft; LV maintains limits always applied and are clearly shown on all schedule documents since at least 2008</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Mr G: when he first took out the policy in 2002 LV told him the valuables and personal possessions limits did not apply to theft claims; LV never informed him this had changed; if he had known limits applied he would have arranged higher cover. LV: limits clearly shown on policy schedule documents; Mr G was told he could change them; £100 paid for complaint handling about how the claim was managed. FOS: no recording or documents available from 2002 inception; standard industry approach is for limits to apply to all claims — it is unlikely Mr G was told limits didn't apply to theft; earliest available documents from 2008 show £5,000 valuables limit; 2015 schedule identical; policy summary explains limits apply; full policy states contents covered up to limits shown on schedule; no exception for theft; Mr G admitted not reading renewal documents sent each year.</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — LV entitled to apply valuables and unspecified personal possessions limits to Mr G's theft claim; no additional payment required beyond what LV had already paid</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Policy limits for specified categories (valuables, unspecified personal possessions) apply to all claims including theft unless the policy explicitly states otherwise — there is no industry standard or practice of limits not applying to theft claims; an unsubstantiated allegation that verbal assurances at inception override clearly-stated schedule limits will not be upheld without supporting evidence, especially where the allegation contradicts standard industry practice; policy limits clearly shown on the schedule and renewal documents bind the policyholder whether or not those documents were read — the obligation to read and understand renewal documents rests with the policyholder; jewellery or valuables exceeding the schedule limit require separate specified item cover to obtain adequate protection</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Recording or documentation from the original 2002 policy inception (not available — earliest LV documents from 2008; the absence of inception records is the central evidential gap; no contemporaneous evidence of what was said about limits at the point of sale)</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>No evidence available from 2002 inception — no telephone recording or documents; Mr G alleges limits were said not to apply to theft but standard industry practice is for limits to apply to all claims; unlikely he was told otherwise; earliest documents from 2008 show £5,000 valuables limit on the schedule; 2015 schedule identical; policy summary and full policy explain limits apply; no exception for theft stated in any document; Mr G admitted not reading renewal documents each year — would have seen and understood limits if he had done; limits fairly applied to his theft claim; LV not required to pay more; £100 voluntarily paid for complaint handling already noted</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>Where a policyholder alleges an oral representation at inception overrides clearly stated policy limits, FOS requires contemporaneous evidence — undocumented telephone conversations from many years before the claim are insufficient to override schedule limits; policy schedules and renewal documents sent each year confirm current limits — policyholders who do not read renewals cannot later claim ignorance of limits shown thereon; handlers should proactively advise policyholders with high-value jewellery to consider whether the valuables sub-limit is adequate and whether separate specified item cover should be arranged</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>IF consumer_alleges_verbal_promise_at_inception_that_limits_do_not_apply AND no_supporting_evidence AND standard_practice_contradicts_allegation THEN FOS_will_not_uphold_allegation; policy_schedule_limits_apply_to_all_claims_including_theft_unless_policy_explicitly_states_otherwise; IF consumer_admits_not_reading_renewal_documents THEN consumer_cannot_claim_ignorance_of_limits_clearly_shown_on_schedule; jewellery_exceeding_valuables_limit_must_be_separately_specified_to_obtain_adequate_cover</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>DRN3351038.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3711750</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>3 Jan 2023</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — primary claim for escape of water (EOW); during RSA-appointed repairers' attendance, jewellery went missing from Miss B's home; Miss B believed RSA's contractors stole it; dispute covers (1) EOW claim handling failures (missed appointments, delays, lost earnings, poor quality work); (2) whether jewellery theft should be dealt with under the EOW claim or as a separate second claim</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Theft by invited contractor — jewellery went missing from home while RSA-appointed painters were attending to carry out escape of water repair works; Miss B believed RSA's repairers were responsible; police investigation was ongoing at time of this FOS decision</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — EOW claim accepted; jewellery theft not declined; RSA agreed to consider theft as a separate second claim with the £200 excess waived (or £200 paid as compensation if theft claim not accepted); dispute concerns whether the theft should be subsumed within the EOW claim and whether RSA's EOW handling compensation is adequate</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Miss B: RSA's repairers clearly stole jewellery on the balance of probabilities; should be dealt with under EOW claim not as a second claim; cash-in-lieu payment too low; having two claims on record is unfair and will increase premiums. RSA: theft is a separate incident from EOW; police investigation ongoing — cannot determine who stole jewellery; £1,740 (lost earnings) + £250 (D&amp;I) is fair for EOW handling failures; cash in lieu must be at RSA repairer rates per policy terms; excess waived for theft claim (or £200 paid as compensation) + £125 for door lock. FOS: not appropriate to determine criminal responsibility — that is a matter for criminal courts; RSA cooperated with police; theft is a separate incident from EOW and two-claim treatment is correct; RSA's EOW compensation package is fair; cash in lieu at RSA repairer rates is policy-compliant; RSA's offer on the theft claim is fair and reasonable.</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — RSA's offer to waive the £200 excess for the theft claim (or pay it as compensation if the theft claim is not accepted) is fair and reasonable; RSA's approach to EOW claim handling compensation and cash-in-lieu settlement is upheld</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>FOS cannot determine whether a specific person committed a theft — that is a criminal matter for the courts; theft of property occurring during contractor attendance for a separate insured peril (escape of water) is a distinct insurable incident and should be treated as a second claim — the fact that the contractors were on site due to the first claim does not merge the two incidents; an insurer's cash-in-lieu settlement is limited to what the insurer's own approved repairers would have charged per standard policy terms; waiving the excess for a theft claim where the insurer's own contractors are the suspected thieves is a fair and reasonable outcome; if police later conclude the insurer's repairers committed the theft, the insurer should then consider whether it is fair to bring the theft claim under the original EOW claim</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>Police investigation outcome (ongoing at time of FOS decision — critical for determining whether RSA's contractors were responsible and whether the theft claim should subsequently be dealt with under the EOW claim); proof of ownership and value of the missing jewellery (required for any theft claim assessment)</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>EOW handling: RSA entitled to use own repairers per policy terms; cash in lieu limited to RSA repairer rates; £1,740 lost earnings + £250 D&amp;I is fair for the significant handling failures (missed appointments, delays, contractor damage); further payment not required. Theft of jewellery: FOS cannot find RSA's repairers stole the jewellery — theft is a criminal matter for courts; theft reported to police; RSA cooperated with police investigation; theft is a separate incident from EOW and two-claim treatment is correct; excess waiver for theft claim (or £200 as compensation if claim not accepted) + £125 for door lock is fair; Miss B cannot be compensated for increased premiums resulting from two-claim recording where the two-claim approach is correct; if police conclude RSA's repairers committed the theft, RSA should reconsider whether to deal with it under the EOW claim at that point</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>Where property goes missing during contractor visits arranged by the insurer for a separate claim, it should be treated as a distinct second claim with its own excess and process — not subsumed into the original claim simply because the same contractors are involved; FOS will not determine criminal responsibility for suspected contractor theft; the insurer should cooperate with the police investigation and consider the theft claim on its own merits; cash-in-lieu settlements should be based on the insurer's own approved repairer rates per policy terms, not the consumer's preferred repairer's quote</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>IF theft_occurs_during_insurer_appointed_contractor_visit THEN treat_as_separate_claim_not_subsumed_within_original_claim; FOS_cannot_determine_criminal_responsibility_for_alleged_contractor_theft; cash_in_lieu_settlement_limited_to_insurer_own_repairer_rates_per_policy_terms; IF insurer_cooperates_with_police_on_contractor_theft_investigation THEN insurer_has_not_acted_unreasonably_in_its_handling</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3711750.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-020</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3764842</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>I.M.S. (London) Limited</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>21 Jul 2023</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Commercial retail insurance (sole trader) — theft of a Vitesse statue at a classic car and autojumble show while trader was packing items into the boot of his car; IMS declined under a policy endorsement (ENDP4639900) requiring either forcible/violent entry or permanently sited security guards for theft cover at exhibition premises; no forced entry occurred and club volunteers do not qualify as permanently sited security guards</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Opportunistic theft at exhibition — Vitesse statue stolen while the sole trader was packing items into the boot of his car at a classic car and autojumble show; no forcible or violent entry; theft occurred during loading in an open outdoor setting</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (sole trader retail insurance — stock and contents at exhibitions)</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Policy endorsement ENDP4639900 requires either (i) forcible or violent entry or (ii) exhibition premises protected by permanently sited security guards for theft cover at exhibitions; no forced entry occurred; club volunteers managing car parks, entrances and issuing wristbands are not 'permanently sited security guards'; event organiser confirmed to the loss adjuster that no paid security guards were used at the event; endorsement conditions not met</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>C (Mr W): club volunteers who managed car parks, entrances and issued wristbands constitute security measures and satisfy the endorsement requirement for permanently sited security guards. IMS: event organiser confirmed no security guards were employed — only club volunteers; volunteers do not meet 'permanently sited security guards' standard; endorsement was added when cover limits were increased — signals requirement for professional security. FOS: accepted no forced entry occurred; considered whether volunteers satisfy 'permanently sited security guards'; volunteers had various responsibilities (car parks, entrances, wristbands) and are not permanently sited professional security staff; exhibitions are high-risk events; endorsement added as condition of increased cover limits — suggests requirement for permanent professional security guards; IMS acted fairly in declining.</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — IMS acted fairly and reasonably in declining the theft claim by relying on the policy endorsement; IMS not required to do anything differently</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>A retail policy endorsement requiring 'permanently sited security guards' at exhibition premises for theft cover (where no forcible/violent entry occurred) means paid, professional security staff permanently stationed at the event — club volunteers with multiple administrative responsibilities (car parks, entrances, wristband issuance) do not meet this standard; exhibitions are recognised as high-risk events for stock theft — endorsements mandating professional security are a reasonable and enforceable insurer risk control; an endorsement added as a condition of increasing cover limits is a deliberate underwriting risk control that must be strictly complied with; the absence of both forcible entry and permanently sited security guards means the endorsement is breached and the claim is excluded</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Full scope of volunteer duties and deployment at the event (assessed by FOS but found insufficient); copy of original endorsement negotiation documents showing the intent behind 'permanently sited security guards' (not needed — FOS satisfied the standard means paid professional security)</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>No forcible or violent entry — accepted by both parties; must therefore consider whether the exhibition premises were protected by permanently sited security guards; event organiser confirmed no paid security guards at event — only club volunteers; volunteers had various responsibilities including car parks, entrances, and wristband issuance and do not satisfy 'permanently sited security guards'; exhibitions are high-risk events so a requirement for professional security is reasonable; endorsement was added when cover limits were increased — signals a deliberate requirement for permanent professional security rather than ad hoc volunteer arrangements; C did not comply with the endorsement; IMS acted fairly and reasonably</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>Commercial traders attending exhibitions must verify their policy endorsements and confirm professional security guard arrangements before each event — a 'permanently sited security guards' requirement is not satisfied by event volunteers with general administrative roles; sole traders should seek written confirmation from event organisers about security arrangements to verify endorsement compliance before attending; endorsements added as conditions of increased cover limits are deliberate high-risk controls that must be strictly met</t>
+        </is>
+      </c>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>IF exhibition_theft_endorsement_requires_permanently_sited_security_guards AND only_volunteer_marshals_present THEN endorsement_not_met_and_theft_claim_excluded; permanently_sited_security_guards_means_paid_professional_security_staff_not_volunteers_with_multiple_responsibilities; IF no_forcible_or_violent_entry AND no_permanently_sited_security_guards THEN exhibition_theft_endorsement_is_breached; IF endorsement_added_as_condition_of_increased_cover_limits THEN endorsement_requirements_are_deliberate_risk_controls_to_be_strictly_applied</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3764842.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Theft Batch 3 (THEFT-021 to THEFT-030)
10 FOS theft decisions appended to Theft_Case_Database.xlsx (30 rows total).
All cases non-core: motor/motorcycle/motorhome/commercial — No Commercial or No Broker Dispute.
Key themes: keys-in-vehicle exclusions, garaging endorsements, Thatcham tracker conditions,
ICOBS 8.1.2(B) causal connection, lost/stolen keys benefit vs full theft section,
NCD misclassification, malicious damage vs self-interested tenant damage.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Theft_Case_Database.xlsx
+++ b/knowledge/case-databases/Theft_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2703,6 +2703,1056 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="120" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>DRN4331324</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Acromas Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>15 Mar 2017</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — car stolen after policyholder left keys in ignition with engine running while visiting a friend for 10–15 minutes; Acromas declined under 'keys in vehicle' exclusion in both Loss or Damage section and General Exceptions; Acromas initially gave misleading information that it would meet the claim, corrected next day; £100 compensation paid for the misleading information</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft — keys left in ignition with engine running while policyholder went into friend's house for 10–15 minutes; car stolen during that absence; policyholder did not intend to leave it unattended but made a conscious decision to go inside</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Policy 'keys in vehicle' exclusion applied — car left unattended with keys in ignition and engine running for 10–15 minutes; exclusion stated in both the Loss or Damage section and General Exceptions of the policy, and in the Certificate of Insurance; Acromas also stated in the policy booklet that Mr M must protect the car from loss; £100 compensation already paid for initial misleading information</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Mr M: didn't intend to leave car unattended; was invited in by friend briefly. Acromas: exclusion clearly applies — keys in ignition while unattended; exclusion sufficiently highlighted in multiple policy sections. FOS: Mr M made a conscious decision to go inside for 10–15 minutes; policy exclusion stated in multiple locations (Loss or Damage section, General Exceptions, Certificate of Insurance); Acromas corrected incorrect information next day; £100 compensation for brief misleading period is fair; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Acromas' decision to decline the theft claim was reasonable; 'keys in vehicle' exclusion sufficiently highlighted; £100 compensation for misleading information was proportionate</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>A 'keys in vehicle' exclusion applies whenever a vehicle is left unattended with keys in the ignition regardless of the policyholder's intention or brevity of absence; the exclusion is sufficiently highlighted when stated in multiple policy sections (Loss or Damage section, General Exceptions, and Certificate of Insurance); where an insurer initially gives misleading information that it will meet a claim but corrects it the next day and pays £100 compensation, the remedy is proportionate; the policyholder's general duty in the policy booklet to protect the vehicle reinforces the exclusion</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>No material missing evidence — facts not in dispute; Mr M accepted he left the car with keys in the ignition for 10–15 minutes while visiting his friend</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>Mr M made a conscious decision to go into his friend's house for 10–15 minutes, leaving the car with keys in the ignition and engine running; policy exclusion applies in exactly these circumstances; exclusion stated in Loss or Damage section, General Exceptions and Certificate of Insurance; Acromas gave misleading information initially but corrected it next day and paid £100; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>A 'keys in vehicle' exclusion is enforceable where the policyholder consciously leaves the vehicle — even briefly — with keys in the ignition; stating the exclusion in multiple policy documents (Loss or Damage section, General Exceptions, Certificate of Insurance) creates a strong case for sufficient disclosure; when an insurer initially gives wrong information about a claim but corrects it within 24 hours, modest D&amp;I compensation (£100) is the appropriate remedy</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>IF keys_left_in_ignition AND vehicle_left_unattended THEN keys_in_vehicle_exclusion_applies_regardless_of_duration_or_stated_intention; IF exclusion_stated_in_multiple_policy_sections_including_certificate THEN exclusion_is_sufficiently_highlighted; IF insurer_gives_misleading_claim_decision_corrects_within_24_hours AND pays_100_compensation THEN remedy_is_proportionate</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>DRN4331324.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="120" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-022</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>DRN4423879</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Liverpool Victoria Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>19 Apr 2018</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Motor (motorcycle) insurance purchased through broker — motorbike stolen; LV declined under garaging endorsement requiring the motorbike to be kept in a 'properly constructed and locked garage'; Mr K's storage area had a brick-frame entrance and metal shutter but rear opened to garden, sides were part timber/plastic or glass, and roof was made of plastic panels; LV could not clearly define 'properly constructed' but assessed physical construction from photographs</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft (motorcycle) — motorbike stolen from storage area that appeared garage-like at the entrance but was structurally inadequate; rear opened to garden, sides non-solid (timber/plastic/glass), roof plastic panels; precise theft method not described</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal motorcycle insurance)</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Policy garaging endorsement required motorbike to be kept in a 'properly constructed and locked garage'; the storage area had a brick-frame entrance and metal shutter but the rear was not secure (opened to garden), sides were part timber/plastic or glass, and the roof was plastic panels per online image provided by LV — not a properly constructed garage</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Mr K: the storage area looks like a garage; LV has not clearly defined 'properly constructed'; endorsement terms are ambiguous. LV and investigator: photos show the area is not secure — rear opens to garden, sides non-solid, roof plastic. FOS: reviewed photos and online image; entrance has appearance of a garage (brick frame, metal shutter) but rear not secure, opens to garden; sides part timber and part plastic/glass; roof plastic panels; not a properly constructed and locked garage; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — LV's decision to decline was reasonable; Mr K's motorbike was not kept in a properly constructed and locked garage as required by the garaging endorsement</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>A 'properly constructed' garage requires full structural integrity on all sides including the rear and roof — an enclosure with an impressive brick-frame entrance and metal shutter does not satisfy the requirement if the rear opens to a garden, sides are non-solid (timber/plastic), and the roof is plastic panels; where a policy endorsement requires a 'properly constructed and locked garage' without defining the term, the ordinary meaning applies: the entire structure must be fully enclosed and secure; the visual appearance of the entrance alone is insufficient if the remainder of the structure is inadequate</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>No material missing evidence — the physical construction of the storage area was assessed from photographs provided by Mr K and online images provided by LV</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Policy schedule included garaging endorsement requiring properly constructed and locked garage; policy does not define 'properly constructed'; reviewed photographs — entrance has brick frame and metal shutter giving appearance of a garage; inside: rear not secure, opens to garden; sides part timber and part plastic/glass; LV also provided online image showing plastic panel roof; not a properly constructed and locked garage; endorsement conditions not met; LV's decision was fair and reasonable; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>When assessing a garaging endorsement, handlers must look beyond the entrance — the rear, side walls and roof must all provide genuine structural security; photographs of all sides (including rear and roof) should be obtained; the absence of a policy definition of 'properly constructed' does not assist the claimant — the ordinary reasonable meaning requires full structural security on all sides</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>IF garaging_endorsement_requires_properly_constructed_locked_garage AND storage_area_has_unsecured_rear_or_non_solid_sides_or_plastic_roof THEN endorsement_not_satisfied; properly_constructed_garage_requires_full_structural_integrity_on_all_sides_including_rear_and_roof; absence_of_policy_definition_of_properly_constructed_means_ordinary_reasonable_meaning_applies</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>DRN4423879.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="120" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4621255</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>20 Mar 2024</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — theft claim accepted and settled by UKI; Mr S raised post-settlement complaints: (1) UKI incorrectly told him he had 4 years' NCD when correct figure was 2 years after the theft claim reduced it; (2) UKI classified the theft claim as 'at fault'; (3) UKI failed to call him back; Mr S has medical conditions and disabilities that heighten his susceptibility to stress; incorrect NCD information caused him to underestimate premium increases with his new insurer</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft — car stolen; circumstances of theft not disputed; all issues in this decision concern post-settlement NCD information error and claim classification rather than the theft circumstances</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — theft claim accepted and settled by UKI; dispute concerns incorrect NCD information given post-settlement and the 'at fault' classification of the theft claim</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Mr S: UKI told him he had 4 years' NCD (wrong — 2 years correct after theft claim reduced it); theft should not be 'at fault' as it was outside his control; T&amp;Cs unclear; medical conditions and disabilities heightened impact of the error. UKI: NCD error acknowledged; 'at fault' classification correct industry practice where no third party to recover from; policy terms clear on NCD reduction; £50 initial compensation offered. FOS: NCD error admitted; 'at fault' classification is correct and policy wording is clear; Mr S's documented medical conditions make the error's impact greater — total compensation of £300 is fair (deducting £50 already paid)</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>UKI must pay Mr S £300 total compensation (deducting sums already paid); 'at fault' classification of the theft claim upheld as correct industry practice; NCD error is upheld as UKI's mistake warranting increased compensation given Mr S's medical conditions</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>A theft claim where no third party can be pursued is correctly classified as a 'fault/bonus-disallowed' claim — the term 'at fault' describes the insurer's inability to recover costs, not the policyholder's culpability; policy terms stating 'if you claim on your policy, we may reduce the NCD' are clear and apply to theft claims; where an insurer misstates NCD information causing a policyholder to underestimate premium increases with a new insurer, compensation must reflect the actual impact — including any documented medical conditions and disabilities that heighten the effect of the error</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>None material on the NCD error — UKI admitted the mistake; the uplift in compensation reflects Mr S's documented medical conditions and their sensitivity to stress</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>'At fault' classification is correct industry practice — insurers record claims as 'at fault' (bonus-disallowed) when there is no third party to pursue; NCD policy terms are clear; NCD error admitted by UKI; Mr S had to notify new insurer and pay more than expected; Mr S has medical conditions seriously impacted by stressful situations — error's impact on him was greater than on most; £50 insufficient; £300 total (net of amount already paid) is fair and reasonable</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>Insurers must verify NCD information before communicating it post-claim, as errors directly affect premiums with the next insurer; a theft claim is correctly classified 'at fault' (bonus-disallowed) in industry databases where no third party can bear the insurer's costs; when assessing compensation for NCD misinformation, policyholders' disclosed medical conditions that heighten susceptibility to financial stress are relevant to the quantum of any award</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>IF theft_claim AND no_third_party_to_recover_from THEN claim_correctly_classified_as_fault_and_NCD_may_be_reduced; IF insurer_misstates_NCD_information_post_settlement THEN compensation_must_reflect_actual_financial_and_emotional_impact; IF policyholder_has_documented_medical_conditions_heightening_impact_of_insurer_error THEN compensation_uplift_is_appropriate</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4621255.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-024</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4800291</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited trading as NIG</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>30 Aug 2024</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Commercial motor trade insurance — vehicle theft claim made October 2023 plus a simultaneous fire damage claim on the same policy; NIG experienced delays and communication issues; M (limited company) failed to provide vehicle keys to NIG for 3+ months; CCTV footage required specialist recovery and was recovered after NIG's final response; NIG offered £350 compensation for handling issues; M disputed NIG's right to require a formal interview and claimed no obligation to provide evidence after 30 days from policy expiry</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft (commercial motor trade) — specific method of theft not described; claim under investigation at time of FOS decision; a second fire damage claim on the same policy was made shortly after the theft claim, adding complication</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (motor trade insurance — not home/contents)</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — claim not declined; dispute concerns NIG's handling delays, its right to require a formal interview as part of the investigation, and the interpretation of the policy's 30-day evidence provision</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>M: NIG has enough information to settle the claim; not obliged to provide evidence more than 30 days after policy expiry; formal interview not contractually required. NIG: M delayed providing keys for 3+ months; CCTV required specialist recovery; simultaneous fire and theft claims warranted detailed investigation; formal interview is reasonable; £350 offered for handling issues. FOS: M caused delays by not providing keys timely; simultaneous fire claim justifies more detailed investigation; one formal interview request is reasonable in complex circumstances; policy 30-day limit applies to when M must provide evidence, not when NIG can request it; £350 adequate for inconvenience; limited company cannot experience distress</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>NIG's offer of £350 compensation for handling delays and communication issues is fair and reasonable; NIG is entitled to require a formal interview before settling the claim; M must engage with the formal interview process</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>A policy clause requiring evidence within 30 days of the loss event imposes a duty on the policyholder to provide evidence promptly — it does not impose a deadline on when the insurer can request evidence; a request for a formal interview is reasonable where simultaneous theft and fire claims exist on the same policy; a limited company cannot claim distress — compensation is limited to inconvenience; a single formal interview request (distinguished from multiple requests) falls within the policyholder's general obligation to provide reasonably required evidence; insurer's claim investigation obligations persist after policy expiry if the claim was made during the policy period</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>CCTV footage content (recovered after NIG's final response); outcome of formal interview with M's director (not yet conducted at time of FOS decision)</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Simultaneous theft and fire claims on same policy justify detailed investigation; M caused delay by not providing keys for over 3 months — no claim decision appropriate until keys provided; CCTV only recovered after final response so reasonable no decision was made; 30-day clause in policy applies to policyholder's duty to provide evidence, not to when insurer can request it; one formal interview is reasonable in complex circumstances; £350 adequate for inconvenience; limited company cannot experience distress; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>Where two serious claims occur close together on the same policy (theft and fire), insurers are entitled to conduct detailed investigations including requesting formal interviews; policyholders who delay providing required evidence cannot subsequently complain about claim delays; a single formal interview request in complex multi-claim circumstances is reasonable; a company complainant cannot receive distress compensation — awards limited to inconvenience</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>IF simultaneous_theft_and_fire_claims THEN more_detailed_investigation_including_formal_interview_is_justified; IF policyholder_delays_providing_required_evidence THEN insurer_not_responsible_for_resulting_delay; policy_30_day_evidence_provision_imposes_duty_on_policyholder_not_deadline_on_insurer; IF complainant_is_limited_company THEN distress_award_not_available_only_inconvenience</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4800291.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="120" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4979740</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Admiral Insurance (Gibraltar) Limited</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>25 Oct 2024</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — home burglary February 2024; Mrs G's car keys stolen and car taken; car recovered by police within one hour with no damage; Mrs G arranged for car lock to be recoded and locks replaced; she wanted to claim under the policy 'lost or stolen keys' benefit (section 2.4: up to £500 reimbursement, no excess, no NCD impact); Admiral insisted on treating as a full theft claim under section 2.1 (excess payable, NCD affected)</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Theft of car keys during home burglary — home broken into while occupants slept; car keys stolen and car taken but recovered by police within one hour with no damage; Mrs G arranged for car lock to be recoded and house and car locks replaced</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — claim not declined; Admiral accepted a claim but insisted on applying section 2.1 (full theft terms with excess and NCD impact) rather than section 2.4 (lost/stolen keys benefit: no excess, no NCD impact, up to £500)</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Mrs G: only claiming for key/lock replacement; car was recovered before she contacted Admiral; section 2.4 does not exclude itself because the car was also stolen. Admiral: section 2.1 must apply because the car was stolen — insisted on full theft terms. Investigator agreed with Mrs G. FOS: car recovered before Mrs G contacted Admiral; Admiral has not dealt with a vehicle theft loss; Mrs G only claims for key/lock replacement under section 2.4; no policy wording prevents section 2.4 from being used in these circumstances; applying section 2.1 with harsher terms is unfair; complaint upheld</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>Admiral must meet Mrs G's claim under section 2.4 of the policy — no excess, no NCD impact, up to £500 reimbursement; Admiral to pay 8% simple interest per annum on reimbursement from date Mrs G paid to date Admiral reimburses; Mrs G must provide proof of payment</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>Where a motor policy provides a distinct 'lost or stolen keys' benefit (no excess, no NCD impact) and the policyholder only claims for key/lock replacement, the insurer must apply that specific benefit rather than the broader theft section — even where the car was also stolen — provided the car has been recovered and no vehicle loss or damage claim is being made; an insurer cannot apply harsher policy terms in place of a specific named benefit unless the policy wording explicitly excludes the benefit in those circumstances; when a vehicle is recovered before the claim is made, the insurer has not dealt with a 'theft claim' for the vehicle and cannot rely on the theft event to override the keys-only benefit</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>None material — dispute was entirely one of policy interpretation; Mrs G must provide proof of payment for Admiral's reimbursement</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>Section 2.4 covers lost/stolen keys with no excess and no NCD impact if claiming only under that benefit; car recovered by police before Mrs G contacted Admiral; no loss or damage to car; Mrs G only claiming for key/lock replacement; Admiral has not had to deal with a vehicle theft loss; applying section 2.1 with excess and NCD impact is unfair when no vehicle loss claim is being made; policy does not exclude section 2.4 where car was also stolen but recovered; complaint upheld; 8% simple interest on reimbursement</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>Handlers must identify the specific policy benefit that actually applies to the consumer's loss — where keys are stolen but the vehicle is recovered undamaged and no vehicle loss/damage claim is made, the 'lost/stolen keys' benefit applies; the mere fact that a vehicle was temporarily stolen does not convert a key-replacement claim into a full theft claim where the vehicle is recovered before the claim is made; policyholders should be informed that claiming under the keys-only benefit preserves their NCD</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>IF consumer_claims_only_for_lost_stolen_keys AND vehicle_recovered_before_claim_made AND no_vehicle_loss_or_damage_claimed THEN lost_stolen_keys_policy_benefit_applies_not_full_theft_section; insurer_cannot_apply_full_theft_terms_if_policy_does_not_explicitly_exclude_keys_benefit_in_theft_circumstances; IF vehicle_recovered_before_insurer_dealt_with_theft THEN insurer_has_not_processed_theft_claim_and_cannot_override_keys_benefit</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4979740.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="120" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5011646</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Mulsanne Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>25 Oct 2024</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — car stolen March 2023; Mulsanne declined because the policy and schedule required a Thatcham-approved tracking device as a condition of theft cover; vehicle had no tracker fitted; Dr M also has a separate complaint about the sales process that led to this policy term (handled separately as a different regulated activity)</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft — car stolen; specific method of entry not described; the policy security requirement (Thatcham-approved tracker) was not met at time of loss</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Policy wording stated theft claims only covered if required security requirements are met; Dr M's schedule specifically required a Thatcham-approved tracking device; no tracker was fitted to the vehicle; security requirement not met; complaint about the sales process is addressed separately as a different regulated activity</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Dr M: when the policy was taken out, he did not agree that the car had a tracker; the sales process was unfair. Mulsanne: policy and schedule clearly require Thatcham-approved tracker for theft cover; no tracker fitted — not disputed. FOS: policy wording and schedule are clear; no tracker fitted — undisputed; sales process complaint is a separate regulated matter handled separately; on this claim-only complaint, Mulsanne applied the policy terms fairly; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Mulsanne fairly and reasonably declined the theft claim; policy terms and schedule clearly required a Thatcham-approved tracking device which was not present</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P27" s="5" t="inlineStr">
+        <is>
+          <t>Where a policy schedule specifically requires a Thatcham-approved tracking device as a condition of theft cover, the absence of any tracker means theft cover does not apply — even if the policyholder disputes the sales process that led to that requirement; FOS treats the sales process complaint and the claim decision complaint as separate regulated activities; on a claim-only complaint, FOS assesses whether the insurer fairly applied the policy terms as they exist, not whether those terms should have been included; a complaint about the fairness of the sales process that generated a policy term does not affect the enforceability of that term in a claim decision</t>
+        </is>
+      </c>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>Whether Dr M was clearly informed at point of sale that a tracker was required (addressed in the separate sales complaint, not in this decision)</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>Policy says theft claims only covered if required security requirements met; schedule specifies Thatcham-approved tracking device; no tracker fitted — not disputed by Dr M; Dr M's concern about the sales process is being handled separately; on the current complaint about the claim decision, Mulsanne applied the policy terms fairly; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S27" s="5" t="inlineStr">
+        <is>
+          <t>A tracker endorsement on a motor policy is an absolute condition of theft cover — there is no dispensation for vehicles where the policyholder disputes having agreed to the requirement during the sales process; FOS treats the sales process complaint and the claim decision complaint as distinct regulated activities; insurers can rely on clear policy schedule terms in a claim complaint even when the sales process is disputed in a parallel complaint</t>
+        </is>
+      </c>
+      <c r="T27" s="5" t="inlineStr">
+        <is>
+          <t>IF policy_schedule_requires_thatcham_tracker AND no_tracker_fitted THEN theft_claim_excluded; sales_process_complaint_is_separate_regulated_activity_from_claim_decision_complaint; IF insurer_applies_clear_policy_schedule_endorsement THEN claim_decline_is_fair_regardless_of_parallel_sales_process_dispute</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5011646.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="120" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5275985</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Wakam</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>5 Apr 2025</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Motor (motorhome) insurance — motorhome stolen from outdoor storage yard; Wakam repudiated the claim citing significant corrosion (rust) in breach of the policy condition 'You shall maintain Your Motorhome in efficient condition'; motorhome later recovered badly damaged; Wakam subsequently conceded it could not fairly rely on mileage discrepancy or misrepresentation grounds; FOS found the rust was not causally connected to the theft under ICOBS 8.1.2(B); £400 D&amp;I compensation ordered</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft (motorhome) — motorhome stolen from outdoor storage yard; specific method of theft not described; vehicle later recovered with extensive internal damage and items stolen from it</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal motorhome insurance)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Policy condition requiring motorhome to be maintained in 'efficient condition' allegedly breached due to significant corrosion (rust) visible on post-recovery inspection; Wakam argued rust was pre-existing and should have been noticed at the last MOT; Wakam also initially relied on mileage discrepancies and possible misrepresentation but later conceded these grounds could not be fairly relied upon</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Mr S: motorhome passed MOT on 31 March 2023 with no advisory notices relating to rust; rust is characteristic of a 30-year-old vehicle stored outdoors; he had invested significantly in the motorhome. Wakam: inspection photos show substantial corrosion from scale rust to penetrating rust; rust of this severity would have been visible at last MOT. FOS: MOT passed March 2023 with no rust advisories; 14 months elapsed between MOT and Wakam's post-recovery inspection; rust may have developed or worsened in that time; even if rust breached the condition, Wakam has not shown causal connection between the rust and the theft (ICOBS 8.1.2(B)); mileage and misrepresentation grounds conceded by Wakam; pre-existing rust deductible from indemnity settlement; £400 D&amp;I; 8% interest from initial rejection</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>Wakam must reconsider the theft claim in line with remaining policy terms and limits, including damage to the motorhome and stolen accessories/equipment; pre-existing rust damage (identified by Wakam's engineer's report) may be deducted from any settlement; 8% simple interest per annum from date of Wakam's initial rejection to date of settlement; £400 D&amp;I compensation for avoidable trouble and upset caused by Wakam's unreasonable handling</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>Under ICOBS 8.1.2(B), a rejection of a consumer policyholder's claim for breach of a policy condition is unreasonable unless the circumstances of the claim are connected to the breach; an insurer cannot rely on a vehicle maintenance condition to repudiate a theft claim without demonstrating causal connection between the breach and the theft itself; a recent MOT pass with no rust advisories is strong evidence that rust visible at post-theft inspection may have developed or worsened after the MOT; a stolen vehicle that is later recovered remains a theft claim in respect of post-theft damage — the insurer cannot reclassify it as an accidental damage total loss claim simply because the vehicle was recovered; pre-existing unrelated damage (rust) may be deducted from any theft indemnity settlement but the claim cannot be fully declined without causal connection to the loss</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>Evidence establishing causal connection between the corrosion and the theft (e.g. that rust around locks facilitated entry) — absent and critical; without this causal link ICOBS 8.1.2(B) prevents reliance on the condition breach to decline the claim</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>Motorhome passed MOT 31 March 2023 with no rust advisories; 14 months before Wakam's post-recovery inspection — rust may have developed or worsened; Wakam cannot persuasively demonstrate causal connection between rust and the theft; ICOBS 8.1.2(B) requires causal connection between breach and loss; mileage and misrepresentation grounds conceded; vehicle remains a theft claim even after recovery; pre-existing rust excluded from settlement; Wakam's handling caused avoidable distress — £400 D&amp;I; 8% interest from initial rejection to settlement date</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>Before repudiating a theft claim on a general vehicle condition clause, insurers must affirmatively establish causal connection between the breach and the theft — ICOBS 8.1.2(B) prevents reliance on unconnected breaches; a recent MOT with no relevant advisories substantially weakens any claim that a defect was pre-existing; post-theft inspection findings must be compared to the last MOT record before asserting a pre-existing breach; the indemnity principle allows pre-existing unrelated damage to be excluded from settlement but does not permit the entire claim to be declined without causal connection to the loss</t>
+        </is>
+      </c>
+      <c r="T28" s="3" t="inlineStr">
+        <is>
+          <t>IF claim_repudiated_for_policy_condition_breach AND breach_not_causally_connected_to_theft THEN repudiation_unreasonable_under_ICOBS_8_1_2_B; IF vehicle_passed_recent_MOT_without_relevant_advisories THEN insurer_cannot_assume_defect_was_pre_existing_without_further_evidence; pre_existing_unrelated_damage_may_be_deducted_from_theft_settlement_but_full_decline_not_permitted_without_causal_connection; stolen_and_recovered_vehicle_remains_theft_claim_for_post_theft_damage</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5275985.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="120" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-028</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>DRN5412255</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Lloyds Bank Insurance Services Limited</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — policy brokered by Lloyds TSB originally voided by underwriter for alleged non-disclosure; Lloyds TSB later admitted the mis-sale and provided 12 months' own-policy cover at the original premium plus £100 D&amp;I compensation; Ms H made a theft claim under the remedial policy (accepted and settled); Ms H subsequently struggled to find affordable renewal insurance in the open market, alleging Lloyds TSB bore ongoing responsibility for higher premiums caused by her theft claim now on record</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Home theft — specific theft circumstances not described in this decision; theft claim was accepted and settled under the remedial Lloyds TSB policy; the dispute concerns the downstream effect on premium costs, not the theft event itself</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — theft claim was accepted and settled during the remedial policy period; dispute concerns whether Lloyds TSB bears ongoing responsibility for higher market premiums resulting from the legitimately-recorded theft claim</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>Ms H: Lloyds TSB as broker mis-sold the original policy; should have offered renewal at the original premium; theft claim on her record causes higher premiums in the market and at renewal; Lloyds TSB should bear responsibility. Lloyds TSB: the mis-sale was fully remedied — 12 months' cover at original premium, £100 D&amp;I, CUE voidance record cleared; theft claim is legitimate and not connected to the original error; premium pricing is each insurer's commercial judgment. FOS: Lloyds TSB fully remedied the mis-sale; CUE voidance record confirmed cleared; theft claim on remedial policy is a legitimate claims record not connected to the original error; market and renewal premium pricing is each insurer's commercial judgment — FOS cannot interfere; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Lloyds TSB appropriately remedied the original policy mis-sale; not responsible for market premium increases arising from the legitimately-made and recorded theft claim</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P29" s="5" t="inlineStr">
+        <is>
+          <t>A broker who mis-sells a policy discharges its remedial obligations by providing equivalent cover at the original premium and paying appropriate D&amp;I compensation — it does not bear ongoing responsibility for how the market prices premiums reflecting a legitimately-made claim on the remedial policy; a theft claim made and accepted on a remedial policy is a legitimate claims record not attributable to the broker's original error once that error has been fully remedied; insurers have commercial discretion to price premiums at renewal based on claims history — FOS cannot interfere; once a CUE voidance/avoidance record is confirmed to have been removed, the broker has no further liability arising from the original policy avoidance</t>
+        </is>
+      </c>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — factual background not disputed; dispute concerned the legal extent of Lloyds TSB's ongoing responsibility after fully remediating the mis-sale</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="inlineStr">
+        <is>
+          <t>Lloyds TSB admitted the mis-sale and offered appropriate remediation (12 months' equivalent cover at original premium, £100 D&amp;I); CUE avoidance record confirmed cleared; Ms H chose not to renew with Lloyds TSB as renewal premium increased — Lloyds TSB has commercial discretion over renewal pricing; open market insurers pricing higher due to theft claim history is their commercial judgment not attributable to Lloyds TSB's original error (which was remedied); the theft claim's existence on Ms H's record is not connected to the mis-sale; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S29" s="5" t="inlineStr">
+        <is>
+          <t>Where a broker mis-sells a policy, full remediation includes correcting any adverse CUE records arising from the mis-sale — once this is done and equivalent cover is provided at the original premium, the broker's obligations are discharged; a theft claim made on a remedial policy creates a legitimate claims record that the policyholder must account for in the open market — this is not attributable to the original broker error; FOS does not interfere in how insurers price premiums at renewal or in the open market</t>
+        </is>
+      </c>
+      <c r="T29" s="5" t="inlineStr">
+        <is>
+          <t>IF broker_provides_remedial_cover_at_original_premium_and_pays_DI_compensation AND corrects_CUE_record THEN broker_has_discharged_mis_sale_remediation_obligations; theft_claim_legitimately_made_on_remedial_policy_creates_valid_claims_record_not_attributable_to_original_broker_error; insurer_renewal_and_market_premium_pricing_is_commercial_judgment_FOS_cannot_interfere</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>DRN5412255.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="120" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5704833</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Complete Cover Group Ltd</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>24 Oct 2025</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance sold through broker Complete Cover Group Ltd — car stolen; insurer declined because the tracker subscription was not activated (tracker device was physically present on the car but the subscription was not continuously active as required by the endorsement); Mr B's representative complained that Complete Cover did not adequately explain the requirement to activate the subscription or how to do so</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft — car stolen; method of theft not described; the endorsement condition not met because tracker subscription was not activated despite the tracker device being physically present</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Insurer declined because tracker subscription was not continuously active at time of theft loss; endorsement required: (1) Thatcham-approved tracking device; (2) subscription continuously active at time of loss; (3) subscription registered in policyholder's or spouse's name; (4) access to subscription account — condition (2) was not met as subscription was not activated</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Mr B's representative: Complete Cover did not draw the tracker subscription activation requirement sufficiently to attention; did not explain steps needed to activate; Mr B believed the subscription came with the car at purchase. Complete Cover: endorsement requirements shown at quotation with mandatory non-prepopulated checkbox acknowledgement; welcome letter clearly stated subscription must be continuously active; policy handbook gave full detail; it is not a broker's responsibility to provide vehicle-specific tracker activation instructions. FOS: requirement disclosed at multiple stages (mandatory checkbox, welcome letter, handbook); clearly presented in the welcome schedule document; it was Mr B's personal responsibility to ensure the subscription was active; broker not required to provide vehicle-specific activation instructions; Mr B could have sought clarification but did not; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Complete Cover adequately disclosed the tracker subscription endorsement requirement at multiple stages; it is not a broker's responsibility to provide vehicle-specific tracker activation instructions</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>A broker adequately discloses a tracker subscription endorsement where: (1) the requirement is shown at quotation with a mandatory non-prepopulated acknowledgement checkbox the consumer must actively tick; (2) the welcome letter explicitly highlights it; (3) the policy handbook provides full detail; a broker is not required to provide vehicle-specific instructions for activating tracker subscriptions — that is the policyholder's personal responsibility; where endorsement requirements are clearly and repeatedly disclosed and the consumer fails to seek clarification, the broker is not liable for the insurer's resulting claim decline</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that Mr B's tracker subscription was or was not active at the time of theft; explanation of why any subscription 'coming with the car' at purchase was not activated or was not registered in Mr B's own name</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>Complete Cover presented tracker endorsement at quotation with a mandatory non-prepopulated checkbox — Mr B had to actively acknowledge it before proceeding; welcome letter clearly stated subscription must be continuously active; policy handbook gave full detail; requirement not hidden — clearly in the welcome policy schedule document; Mr B's representative said he thought subscription came with the car — Complete Cover is not responsible for this assumption; broker not required to provide vehicle-specific activation steps for each customer type; Mr B could have contacted Complete Cover for clarification but did not; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>Brokers can satisfy tracker endorsement disclosure obligations through a combination of mandatory acknowledgement at quotation, clear welcome letter and detailed policy handbook; policyholders bear personal responsibility for ensuring tracker subscriptions are continuously active — this includes verifying that any subscription 'coming with the car' is activated and registered in the correct name; a policyholder who does not seek clarification on endorsement requirements cannot later hold the broker responsible for a resulting claim decline</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>IF tracker_endorsement_disclosed_at_quotation_via_mandatory_non_prepopulated_checkbox AND welcome_letter_and_handbook_also_reference_requirement THEN broker_has_adequately_disclosed_endorsement; IF consumer_fails_to_activate_tracker_subscription AND no_evidence_of_seeking_clarification THEN broker_not_liable_for_resulting_claim_decline; broker_not_required_to_provide_vehicle_specific_tracker_activation_instructions</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5704833.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="120" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-030</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5852242</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited trading as NIG</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2025</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Commercial property insurance — insolvent tenant (tenant two) vacated a commercial let property after becoming insolvent, making unauthorised alterations (partial redecoration, removal of light fixtures causing small holes, removal of aluminium kitchen sheeting) and removing fixtures and fittings; J (limited company landlord) claimed approximately £14,000 for malicious damage and approximately £8,300 for loss of rent; UKI declined — tenant's actions did not constitute 'malicious damage'; FOS agreed; no formal theft claim for removed items was ever submitted to UKI</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Removal of fixtures and fittings by insolvent departing commercial tenant — tenant two vacated after insolvency; made unauthorised changes (partially painted walls, removed light fixtures, removed aluminium kitchen cladding, possibly removed coffee machine); no forced entry; tenant had legitimate access to the property under the lease</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (commercial let property insurance — not home/contents)</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Damage caused by an insolvent tenant vacating and making unauthorised alterations does not constitute 'malicious damage' — malicious damage requires deliberate intention to cause harm directed at the insured or the property; tenant's actions were more consistent with self-interest or refurbishment purposes than with spite or ill will toward J; without an accepted insured event, the loss of rent claim cannot be pursued; no formal theft claim was made to UKI so FOS cannot direct consideration of one</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>J: tenant made unauthorised alterations and removals causing £14,000 damage constituting malicious damage — actions were intentional and caused financial harm; tenant has history of insolvency and not paying staff showing bad character. UKI: 'malicious' requires deliberate intent to cause harm — breach of lease insufficient. Investigator: agreed not malicious damage; recommended UKI consider a theft claim for removed items. FOS: damage not malicious — tenant acting in self-interest not with ill will toward J; partial redecoration consistent with refurbishment; small holes from light fixtures not evidence of intent to harm; aluminium cladding partially left on-site — more consistent with refurbishment than malice; tenant insolvency history does not establish intent to harm J; neglect or acting without care ≠ malicious damage; FOS cannot direct insurer to consider theft claim not formally made or complained about; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — UKI fairly declined the malicious damage claim; FOS will not require UKI to consider a theft claim that was never formally made as part of this complaint; J should make a formal theft claim to UKI</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P31" s="5" t="inlineStr">
+        <is>
+          <t>'Malicious damage' under a commercial property policy requires deliberate intention to cause harm to the insured property or the insured landlord — breach of tenancy agreement and unauthorised alterations are insufficient without positive evidence of spite or ill will directed at the insured; acting without care, or neglect, does not evidence malicious damage unless there is also deliberate intent to cause harm; a tenant acting in its own interests (removing items for use elsewhere, refurbishment) is not acting maliciously even if this causes financial harm to the landlord; loss of rent cover depends on an accepted insured event being established; FOS can only consider complaints about claims formally made and declined or ignored by the insurer — it cannot require an insurer to consider a claim never formally submitted</t>
+        </is>
+      </c>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>Evidence of deliberate intent to harm J by tenant two (absent — all actions appear self-interested); formal theft claim submitted to UKI and UKI's response (not before FOS; J directed to make this claim directly to UKI)</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>Policy covers 'theft and malicious damage by tenant'; malicious damage means damage with deliberate intention to cause harm; partial redecoration consistent with refurbishment not malice; small holes from light fixture removal not evidence of intent to harm; aluminium sheeting partly left on site — more consistent with refurbishment; tenant removing items for another business shows self-interest not ill will; tenant insolvency history does not establish intent to harm J; neglect or acting without care ≠ malicious damage; no accepted insured event so no loss of rent; no formal theft claim made or complained about — FOS cannot review what was never before the insurer as a complaint; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S31" s="5" t="inlineStr">
+        <is>
+          <t>Landlords whose commercial tenants cause damage on vacating must formally make both a malicious damage claim and a separate theft claim — failing to formally make a theft claim means FOS cannot consider it; the 'malicious' element in a commercial property policy requires positive evidence of spite or ill will — significant financial harm to the landlord alone is insufficient; handlers should distinguish between damage serving the tenant's interests (acting without care) and damage intended to harm the landlord (malicious)</t>
+        </is>
+      </c>
+      <c r="T31" s="5" t="inlineStr">
+        <is>
+          <t>IF tenant_causes_damage_or_removes_items_on_vacating AND actions_serve_tenants_own_interests THEN malicious_damage_cover_does_not_apply; malicious_damage_requires_deliberate_intent_to_cause_harm_not_merely_breach_of_tenancy_or_financial_harm_to_landlord; IF loss_of_rent_claimed AND no_accepted_insured_event THEN loss_of_rent_claim_cannot_proceed; FOS_cannot_direct_insurer_to_consider_theft_claim_not_formally_made_and_not_complained_about</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5852242.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Theft Batch 4 (THEFT-031 to THEFT-039) — Theft database complete at 39 rows
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Theft_Case_Database.xlsx
+++ b/knowledge/case-databases/Theft_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3753,6 +3753,951 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="120" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5901721</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>5 Dec 2025</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — car stolen September 2023; Aviva declined to process the theft claim as the policy required an Aviva-approved tracking device to be fitted, in operation, and with subscription maintained; Mr S initially denied having a tracker then claimed he did; named driver Mrs K confirmed in a September 2023 call that a tracker was purchased but was never set up or installed in the car; invoice produced did not specify a tracker; app screenshots showed a basic device not registered to the insured car; secondary complaints concern automatic policy renewal (£75 D&amp;I awarded but not paid), being told to keep paying premiums until theft claim resolved, and whether the premium refund was correctly backdated</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft — car stolen 16 September 2023; method of theft not described; dispute centres on whether the policy tracker condition was satisfied at the time of theft</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Policy clause required an Aviva-approved tracking device to be fitted, in operation, and with subscription maintained at the time of theft; Mr S could not demonstrate the tracker was fitted and working; named driver Mrs K confirmed in a phone call that the tracker was bought but was not set up or installed in the car</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Mr S: claimed to have a tracker; produced dealership invoice for £500 (did not specify tracker) and screenshots of a tracker app. Mrs K: confirmed in September 2023 call that tracker was bought but didn't work and wasn't set up or installed. Aviva: app screenshots showed basic device not shown to be registered to Mr S' car or any car. FOS: Mrs K's own admission is clear evidence the tracker was not fitted and working; Aviva correctly declined the theft claim; automatic renewal error acknowledged — £75 D&amp;I not yet paid and must be paid now; £50 D&amp;I for not responding to backdating email confirmed paid; premium refund correctly backdated to October 2023 (date of Aviva's claim decision); complaint not upheld save for outstanding £75 payment</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Aviva correctly declined Mr S' theft claim as he could not show a working Aviva-approved tracker was fitted as required by the policy; Aviva must pay the outstanding £75 compensation it had already committed to for automatically renewing the policy against Mr S' instructions</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr">
+        <is>
+          <t>A motor policy requiring an Aviva-approved tracking device 'fitted, in operation, and with subscription maintained' is enforceable as a condition precedent to theft cover — the policyholder must demonstrate the tracker was operational at the time of theft; a dealership invoice that does not identify a tracking device and app screenshots not registered to the insured vehicle do not satisfy the tracker condition; where the named driver has confirmed in a recorded call that the tracker was purchased but not set up or installed, that admission is sufficient to uphold the insurer's decision not to pay the theft claim; an insurer should not require a policyholder to continue paying monthly instalments as a condition of processing a theft claim — remaining premium can be deducted from any claim payment; a premium refund following policy cancellation should be backdated to the date the insurer made its decision on the theft claim, not before, as the policyholder had the benefit of third-party liability cover up to that date</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that the tracker was specifically fitted to and registered to Mr S' car and that its subscription was maintained at the time of theft (absent and decisive — Mrs K's own statement confirmed it was not set up or installed)</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>Mrs K confirmed in a September 2023 call that Mr S bought a tracker but it didn't work and wasn't set up or installed in the car; subsequent dealership invoice for £500 did not specify it was for a tracker; app screenshots showed a basic tracking device not registered to Mr S' car or any car; on balance no working tracker was fitted as required by the policy; Aviva was entitled to decline the theft claim; telling Mr S to continue paying instalments was not wrong in principle (premium is payable upfront — instalments are a concession; remaining premium would have been deducted from any claim payment); Aviva adviser wrongly said claim wouldn't be paid if premium stopped but no compensation warranted; premium refund correctly backdated to October 2023 (date of claim decision) — Mr S had the benefit of third-party liability cover until then; £50 D&amp;I for not responding to backdating email confirmed paid; £75 D&amp;I for auto-renewal committed but not paid — must be paid now</t>
+        </is>
+      </c>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>When a policy requires a tracker as a condition of theft cover, handlers must obtain evidence that the device was (1) specifically fitted to the insured vehicle, (2) in operation, and (3) had an active subscription at the time of theft — a generic invoice and app screenshots without vehicle registration proof are insufficient; a named driver's own admission in a call that the tracker was not set up is strong evidence the condition was not met and should be recorded and relied upon; all D&amp;I compensation committed by the insurer must be paid promptly — failure to pay previously committed compensation compounds the complaint and requires FOS to direct payment</t>
+        </is>
+      </c>
+      <c r="T32" s="3" t="inlineStr">
+        <is>
+          <t>IF motor_policy_requires_tracker_fitted_in_operation_with_active_subscription AND policyholder_cannot_demonstrate_tracker_registered_to_insured_vehicle AND named_driver_confirms_tracker_not_set_up THEN tracker_condition_not_met_and_theft_claim_excluded; dealership_invoice_not_specifying_tracker_and_app_screenshots_not_registered_to_vehicle_are_insufficient_tracker_evidence; IF claim_declined_and_policy_cancelled THEN remaining_premium_should_be_deducted_from_claim_payment_not_collected_as_condition_of_processing; premium_refund_backdated_to_claim_decision_date_not_date_of_theft_as_policyholder_had_benefit_of_third_party_cover_until_then</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5901721.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="120" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-032</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>DRN5939533</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Zurich Insurance PLC</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>24 Jul 2017</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Home contents insurance — Mr and Mrs G's domestic employee stole multiple items of jewellery from their home over at least two separate occasions; one item was noticed missing in November 2011 and five further items were reported stolen in February 2012; Zurich recorded two separate theft claims and applied two excesses; Mr and Mrs G argued all thefts were committed by the same person (their employee) and should be treated as one claim</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Theft by trusted domestic employee — employee had access to the home and stole jewellery on at least two separate occasions: one item taken no later than November 2011 and at least one item taken in February 2012; five further items reported missing on the same day as the February 2012 theft with unknown specific dates</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — both theft instances were accepted and paid by Zurich; dispute concerns whether two separate excesses were correctly applied by recording the thefts as two claims rather than one</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>Mr and Mrs G: all items were taken by the same person (their employee) — should be one claim; FOS Technical Helpdesk had advised their broker that FOS would generally treat this as one claim. Zurich: items were taken at different times — at least two separate theft occasions; could reasonably have recorded six separate claims but chose to treat as two. FOS: Technical Helpdesk advice was general guidance only and not binding on this specific case; items were taken at different times (November 2011 and February 2012 are distinct occasions); same perpetrator does not collapse multiple theft occasions into one claim event; Zurich's two-claim recording was fair and actually favourable (could have recorded up to six); complaint not upheld</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Zurich correctly recorded two separate theft claims as items were taken on at least two different occasions; the same perpetrator does not make multiple theft incidents a single claim; Zurich acted generously in recording only two claims rather than up to six</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P33" s="5" t="inlineStr">
+        <is>
+          <t>Multiple thefts by the same perpetrator do not constitute a single theft claim event if the items were taken on different occasions — each separate occasion of theft is a distinct claim to which a separate excess applies; the number of claim events is determined by the number of distinct theft occasions, not the number of items stolen or the identity of the perpetrator; the FOS Technical Helpdesk's general guidance to a broker about how FOS approaches a type of case is not binding on the ombudsman's determination of the specific complaint; where an insurer cannot pinpoint the exact dates of all thefts but can identify at least two distinct occasions, recording the minimum identifiable number of claim events is fair; same proximate cause (same person) does not determine the number of claim events — timing and occasion of each theft do</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Specific dates for all six missing items (only November 2011 and February 2012 occasions were clearly established) — absence of dates supported Zurich's decision to record two rather than up to six separate claims</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>Items were taken at different times — November 2011 and February 2012 are at least two separate theft incidents; same perpetrator does not make it one claim event; Technical Helpdesk gave general guidance not a specific ruling on this case and had not seen all the evidence; Zurich could reasonably have recorded up to six separate claims but fairly chose to treat as two; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S33" s="5" t="inlineStr">
+        <is>
+          <t>When a policyholder reports multiple items stolen by the same person over an extended period, handlers must identify and record each distinct theft occasion as a separate claim event — the number of identified occasions (not items) is the basis for claim counting; where dates of some thefts are uncertain, recording the minimum number of clearly identifiable occasions rather than the maximum is a reasonable and favourable approach; claims handlers must not conflate 'same perpetrator' with 'same incident' — they are different concepts</t>
+        </is>
+      </c>
+      <c r="T33" s="5" t="inlineStr">
+        <is>
+          <t>IF multiple_items_stolen_by_same_person AND thefts_occurred_on_different_occasions THEN each_occasion_constitutes_separate_claim_event_and_separate_excess_applies; same_perpetrator_does_not_make_multiple_theft_occasions_into_one_claim; IF exact_dates_of_some_thefts_unknown THEN recording_minimum_number_of_confirmed_occasions_is_fair_and_favourable; fos_technical_helpdesk_guidance_is_general_and_not_binding_on_specific_complaint_outcome</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>DRN5939533.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="120" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5954307</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Advantage Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>7 Jan 2026</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Motor insurance — Mr M purchased a policy in March 2025 and made a claim in September 2025; Advantage discovered he had failed to disclose a theft claim from 28 February 2025 (less than one month before policy inception) when Miss M (named driver) took out the policy and answered 'no' to a clear question asking about all motor accidents, claims or losses in the past 5 years including unsettled claims; Advantage applied a CIDRA proportionate settlement at 71%</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft — vehicle subject to September 2025 claim; method of theft not described; a prior undisclosed motor theft claim from 28 February 2025 triggered the CIDRA proportionate settlement dispute</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — claim not declined; Advantage applied a CIDRA proportionate settlement at 71% based on the ratio of premium actually paid (£1,401.47) to the premium that should have been charged had the prior theft claim been disclosed (£1,975.21); careless misrepresentation classified as a qualifying misrepresentation</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Miss M: the question was ambiguous; she was going through a very difficult personal period and any error was a genuine mistake not a failure to take reasonable care; she was not aware the prior unsettled claim had to be declared. Advantage: prior theft claim from 28 February 2025 was not declared; would have charged a higher premium if disclosed. FOS: the question is clear and explicitly states it includes unsettled claims; the prior theft claim occurred less than one month before policy inception — a reasonable person would have declared it; personal difficulties acknowledged but do not override failure to take reasonable care; misrepresentation is qualifying (Advantage would have charged more); careless misrepresentation; 71% proportionate settlement is fair</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Advantage correctly identified a careless qualifying misrepresentation under CIDRA; proportionate settlement at 71% (£1,401.47 / £1,975.21) is fair and reasonable</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>Under CIDRA, an insurer may settle a claim proportionately where: (1) the consumer failed to take reasonable care not to make a misrepresentation; (2) the misrepresentation is qualifying (the insurer would have offered the policy on different terms or not at all); and (3) the misrepresentation was careless; a clear disclosure question that explicitly includes unsettled claims means that a consumer who fails to declare a motor claim made less than one month before policy inception has not taken reasonable care, regardless of personal circumstances at the time; the CIDRA proportionate settlement ratio is calculated as: (premium actually paid) divided by (premium that should have been charged), applied to the claim settlement; personal difficulties at the time of taking out a policy are relevant context but do not automatically constitute a defence to a careless misrepresentation</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>No material missing evidence — undisclosed theft claim confirmed by Advantage; premium differential supported by underwriting evidence; CIDRA analysis straightforward on the facts</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="inlineStr">
+        <is>
+          <t>Question was clear and explicitly included unsettled claims; prior theft claim occurred 28 February 2025 — less than one month before March 2025 policy inception; a reasonable person in this position would have declared it; Miss M's difficult personal circumstances are acknowledged but do not override the failure to take reasonable care; misrepresentation is qualifying (Advantage would have charged more — £1,975.21 vs £1,401.47 actually charged); Advantage treated the misrepresentation as careless — appropriate; CIDRA entitles Advantage to pay 71% of the claim; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>CIDRA proportionate settlement is the correct remedy for a careless misrepresentation where the insurer would have charged a higher premium — calculate the ratio of premium paid to premium that should have been charged and apply it to the claim settlement; a disclosure question that explicitly names unsettled claims removes any ambiguity — even a claim made days before policy inception must be declared; a consumer's difficult personal circumstances at the time of taking out a policy are relevant context but do not automatically constitute a defence to careless misrepresentation</t>
+        </is>
+      </c>
+      <c r="T34" s="3" t="inlineStr">
+        <is>
+          <t>IF consumer_fails_to_disclose_prior_motor_claim_when_buying_motor_policy AND question_explicitly_includes_unsettled_claims THEN failure_to_disclose_is_careless_misrepresentation; IF CIDRA_qualifying_misrepresentation_is_careless AND insurer_would_have_charged_higher_premium THEN proportionate_settlement_equals_premium_paid_divided_by_premium_that_should_have_been_charged; prior_motor_claim_less_than_one_month_before_policy_inception_must_be_declared_regardless_of_settlement_status; personal_difficulties_at_time_of_application_are_relevant_context_but_do_not_negate_duty_of_reasonable_care</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5954307.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="120" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-034</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>DRN6242378</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Covea Insurance plc</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Commercial motor insurance taken out through a broker — Mr M's vehicle suffered what appeared to be fire damage (found to be an electrical fault not covered under the policy); Covea voided the policy when it discovered Mr M had not disclosed a previous vehicle theft claim made two years earlier that was subsequently withdrawn after the vehicle was recovered with no damage; the broker had asked whether Mr M had any motoring incidents, accidents or claims including theft in the last 5 years whether or not a claim was made; Mr M believed a withdrawn claim with no payment did not need to be disclosed; dispute before FOS limited to the voidance (vehicle disposal complaint withdrawn by Mr M)</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable to the current claim — the claim before Covea was for fire/electrical fault damage not theft; the prior theft referenced was a vehicle theft two years earlier that was reported to the insurer and then withdrawn when the vehicle was recovered with no damage</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (commercial motor insurance — not home/contents)</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>Broker asked clear question covering all motoring incidents including theft whether or not a claim was made; Mr M failed to disclose a previous vehicle theft claim made two years earlier (withdrawn after vehicle recovery with no damage); Covea voided the policy on non-disclosure grounds; fire/electrical fault damage was separately not covered under the policy terms regardless of voidance</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>Mr M: genuinely believed a withdrawn claim with no payment did not need to be disclosed; didn't claim so shouldn't count. Covea: clear question asked; non-disclosure was deliberate or reckless; even notification-only disclosure would have increased the premium. Adjudicator: withdrawn claim was a notification-only incident not a settled claim; Covea would still have insured Mr M at slightly increased premium; voidance was unfair; fire/electrical fault claim correctly declined; recommended voidance removal and £200 compensation plus salvage amounts for disposal. FOS: Mr M was asked a clear question and the withdrawn claim should have been disclosed as an incident; non-disclosure was not deliberate or reckless; Covea would still have insured Mr M had it been disclosed as a notification-only incident (at slightly increased premium); full voidance was disproportionate and unfair; fire/electrical fault claim correctly declined regardless; complaint upheld in part</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>Covea to remove the voidance from Mr M's record and pay £200 compensation for the distress and inconvenience caused by the unfair voidance; fire/electrical fault claim correctly declined as not a covered peril — no remedy for that element</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P35" s="5" t="inlineStr">
+        <is>
+          <t>An insurer cannot void a policy for non-disclosure of an incident unless: (1) the consumer was asked a clear question; AND (2) had the true facts been disclosed, the insurer would not have offered insurance on the same terms or at all; where the insurer would still have offered insurance (at a higher premium) had the withdrawn claim been disclosed as a notification-only incident, a full voidance is disproportionate — the correct remedy is a premium adjustment not voidance; a withdrawn theft claim where no payment was made is nonetheless a disclosable incident where the broker's question asks about all motoring incidents including theft regardless of whether a claim was made; failure to disclose a withdrawn claim that the policyholder genuinely believed was not disclosable is careless not deliberate or reckless</t>
+        </is>
+      </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>Covea's underwriting evidence as to what premium would have been charged had Mr M disclosed the withdrawn theft claim as a notification-only incident (adjudicator obtained and reviewed — confirmed Covea would still have offered cover at a slightly increased premium)</t>
+        </is>
+      </c>
+      <c r="R35" s="5" t="inlineStr">
+        <is>
+          <t>Mr M was asked a clear and unambiguous question by his broker covering all incidents including theft whether claimed or not; the withdrawn theft claim was an incident that should properly have been disclosed; Mr M's belief it was not disclosable is understandable but non-disclosure was not deliberate or reckless; Covea's underwriting criteria show it would still have insured Mr M had the incident been disclosed as notification-only at a slightly increased premium; full voidance was therefore disproportionate and unfair; fire/electrical fault damage is separately not covered under the policy regardless; Covea to remove voidance and pay £200 D&amp;I compensation</t>
+        </is>
+      </c>
+      <c r="S35" s="5" t="inlineStr">
+        <is>
+          <t>A full policy voidance is only appropriate where the insurer demonstrates it would not have offered cover at all had the true facts been disclosed — where it would have offered cover at a higher premium, the correct remedy is a premium adjustment; handlers must check underwriting criteria before voiding for non-disclosure; a withdrawn claim where the vehicle was recovered with no payment is still a disclosable incident where the question asks about all incidents including theft regardless of whether a claim was made</t>
+        </is>
+      </c>
+      <c r="T35" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_would_still_have_offered_cover_at_higher_premium_had_true_facts_been_disclosed THEN full_voidance_is_disproportionate_and_only_premium_adjustment_is_permitted; IF policy_question_asks_about_all_incidents_including_theft_whether_claimed_or_not THEN withdrawn_theft_claim_is_disclosable_regardless_of_no_payment; non_disclosure_of_withdrawn_claim_policyholder_believed_undisclosable_is_careless_not_deliberate; voidance_requires_proof_insurer_would_not_have_offered_insurance_at_all_not_merely_on_different_terms</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>DRN6242378.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="120" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>DRN6596319</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>UK General Insurance (Ireland) Limited</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2 Oct 2015</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance arranged by telephone May 2013 — Mr B disclosed a legal expenses claim but failed to disclose a prior home theft claim; made a claim under the policy January 2014; UK General cancelled the policy from the start date when it discovered the undisclosed theft claim, stating it would not have offered insurance had the theft claim been disclosed; Mr B argued he forgot about the theft claim and that disclosing a larger legal expenses claim should have covered his obligation</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Home theft — specific circumstances of the prior theft claim not described in this decision; the dispute concerns non-disclosure of that prior theft claim when purchasing home insurance in May 2013; the January 2014 claim type is also not specified</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Undisclosed prior home theft claim — UK General's underwriting criteria show it would not have offered Mr B insurance had the theft claim been disclosed; Mr B failed to disclose the theft claim during the application call despite clear and unhurried questions asking about any home insurance claims and reported losses; answered the claims question by referencing only his legal expenses claim and confirmed no home insurance claims existed when a follow-up question was asked</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Mr B: forgot about the theft claim; disclosed the bigger legal expenses claim; questions were unclear; advisor did not take sufficient care; now having difficulty getting insurance. UK General: clear questions asked about all home insurance claims and losses; theft claim would have made a difference to the offer of insurance; Mr B's answers confirmed no home insurance claims. FOS: clear and unhurried questions were asked about any home insurance claims or reported losses; the word 'any' meant all claims not just the biggest; Mr B answered 'no, but' and mentioned only the legal expenses claim; a follow-up question confirmed no home insurance claims — this should have prompted disclosure of the theft claim; UK General's underwriting criteria show the theft claim would have prevented an offer of insurance; legal expenses policy was with a different underwriter so its claims did not affect UK General's home insurance underwriting criteria; Mr B acted carelessly not deliberately; UK General fairly cancelled the policy from inception</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — UK General fairly and reasonably cancelled Mr B's home insurance policy from inception; Mr B failed to take reasonable care to disclose a prior home theft claim despite clear and unhurried questions being asked during the application call</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>A policyholder asked a clear and unhurried question about 'any' home insurance claims or reported losses must disclose all relevant prior claims — disclosing one (larger) claim does not discharge the obligation to disclose all claims; a follow-up confirmation question ('as long as there were no claims on the home insurance itself or reported losses…is that right') reinforces the duty to disclose and if answered incorrectly does not assist the policyholder; forgetting a prior theft claim when answering a clear question is careless misrepresentation not an absence of misrepresentation; where the insurer demonstrates it would not have offered cover had the prior theft claim been disclosed, cancellation from inception is proportionate and fair; home insurance and legal expenses insurance arranged in the same call may be with different underwriters — the underwriting criteria for each apply independently and a claim under one does not affect underwriting eligibility under the other</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>Specific details of the prior theft claim (amount, circumstances, date) — absent but UK General's underwriting criteria confirmed that a theft claim of Mr B's amount would have made a difference to their decision to offer insurance</t>
+        </is>
+      </c>
+      <c r="R36" s="3" t="inlineStr">
+        <is>
+          <t>UK General asked clear and unhurried questions about any home insurance claims or losses; Mr B answered 'no, but' and described only his legal expenses claim; a follow-up question confirmed no home insurance claims — Mr B confirmed it was fine; legal expenses policy was with a different underwriter — UK General's home insurance underwriting criteria did not take legal expenses claims into account; a theft claim in Mr B's amount would have made a difference to UK General's offer of insurance; Mr B didn't act deliberately but acted carelessly; UK General fairly cancelled the policy from inception; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S36" s="3" t="inlineStr">
+        <is>
+          <t>When assessing non-disclosure in home insurance, handlers must specifically check whether the insurer's underwriting criteria treat the undisclosed claim as a difference-maker — not all undisclosed claims warrant voidance; where a consumer discloses one claim but omits another during the same call, the insurer can rely on a clear follow-up question that the consumer confirms negatively; a policyholder who mentions a claim under one product (legal expenses) arranged in the same call does not thereby discharge disclosure obligations under a separate product (home insurance) sold by a different underwriter</t>
+        </is>
+      </c>
+      <c r="T36" s="3" t="inlineStr">
+        <is>
+          <t>IF policyholder_asked_clear_question_about_any_home_insurance_claims AND fails_to_disclose_prior_theft_claim THEN non_disclosure_is_at_minimum_careless; IF insurer_demonstrates_undisclosed_prior_theft_claim_would_have_prevented_offer_of_cover THEN cancellation_from_inception_is_fair; disclosing_larger_claim_under_different_product_in_same_call_does_not_discharge_disclosure_of_smaller_claim_under_home_insurance; legal_expenses_claims_do_not_affect_home_insurance_underwriting_criteria_when_policies_are_with_different_underwriters</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>DRN6596319.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="120" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-036</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>DRN6785039</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance commenced online March 2010 — Mr B made a theft claim December 2011 and a fire damage claim March 2012; RSA checked an external claims database and discovered Mr B had four previous claims (March 2009, August 2009, October 2009, January 2010) but had only disclosed one (October 2009) in the online application; RSA voided the policy from March 2010 and sought reimbursement of £1,486.22 it had already paid toward the December 2011 theft claim; Mr B disputed that the application was made online (claiming it was by telephone) and that he had disclosed all claims</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Home theft — specific circumstances of the December 2011 theft claim not described; RSA partially settled the claim before discovering the non-disclosure and avoiding the policy</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Non-disclosure of three of four previous claims (March 2009, August 2009, January 2010) made within three years of policy inception — only October 2009 claim was disclosed; online application asked clearly for all claims in the previous three years; RSA demonstrated it would not have offered cover if all four previous claims had been disclosed; RSA also sought reimbursement of £1,486.22 already paid toward the December 2011 theft claim</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>Mr B: application was made by telephone not online; disclosed all claims during the telephone call; RSA's online application documentation is inaccurate; Mr B does not complete application forms himself. RSA: online application exists in Mr B's name in March 2010 showing only one claim disclosed; IP address traced to Mr B's area; four prior claims found on external database at time of fire claim investigation. FOS: balance of probabilities the application was made online — online application record exists, IP address is consistent with Mr B's area, and Mr B cannot provide telephone records; question about previous claims was clear; failure to disclose three claims was inadvertent; RSA demonstrated it would not have offered cover if all four claims disclosed — voidance is reasonable; RSA chose not to check external database at inception — unreasonable to now pursue reimbursement of claims paid during the policy period; RSA accepted it will not pursue the £1,486.22; complaint upheld in part</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>RSA required not to pursue Mr B for reimbursement of its outlay of £1,486.22 in respect of the December 2011 theft claim; no other award — voidance stands, theft and fire claims are not paid, no compensation awarded</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P37" s="5" t="inlineStr">
+        <is>
+          <t>Where a consumer inadvertently fails to disclose previous claims in response to a clear question on an insurance application, this service will generally expect an insurer to apply a proportionate response — where the insurer demonstrates it would not have offered cover at all, avoidance from inception is proportionate; an insurer that chooses not to check a policyholder's external claims database at inception cannot subsequently seek reimbursement of claim payments made during the policy period when it later avoids the policy — the delay in checking is the insurer's own commercial decision and the resulting cost cannot be transferred to the policyholder; where an application method (online vs telephone) is disputed and there is evidence of both an online application record and subsequent phone calls (none of which concerned prior claims disclosure), the balance of probabilities test is applied — an online application record in the consumer's name supported by an IP address consistent with their location outweighs an unverified claim of telephone disclosure not supported by any telephone records; renewal documents listing disclosed claims constitute evidence of the claims history maintained at each renewal</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>Evidence of a telephone call at policy inception during which Mr B disclosed all four prior claims — absent; no telephone records provided by Mr B to support the telephone disclosure claim; RSA traced four calls from Mr B's landline but all post-inception and none concerned prior claims</t>
+        </is>
+      </c>
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Balance of probabilities — online application made; online question asked clearly for all claims in previous three years; only October 2009 claim of four was disclosed; failure to disclose three other claims was inadvertent; RSA demonstrated it would not have offered cover if all four disclosed — avoidance from inception was reasonable; RSA chose not to check external database at application inception — unreasonable to pursue reimbursement of claim payments made during the policy period; RSA already accepted it would not pursue the £1,486.22; upheld in part — only remedy is that RSA must not pursue reimbursement; no compensation, voidance stands</t>
+        </is>
+      </c>
+      <c r="S37" s="5" t="inlineStr">
+        <is>
+          <t>Insurers who do not conduct external claims database checks at inception take on the risk that they have paid claims they cannot recover if they later discover non-disclosure and avoid the policy — this cost cannot be transferred to the policyholder after the fact; where a dispute arises about whether an application was made online or by telephone, the insurer's burden is to demonstrate on the balance of probabilities that the documented online application is authentic; a claimed telephone disclosure that cannot be supported by any telephone records is unlikely to displace a contemporaneous online application record in the consumer's name</t>
+        </is>
+      </c>
+      <c r="T37" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_chooses_not_to_check_external_claims_database_at_inception AND later_discovers_non_disclosure_and_avoids_policy THEN insurer_cannot_recover_claim_payments_made_during_policy_period; IF online_application_record_exists_in_policyholders_name_and_IP_address_matches_policyholders_area THEN balance_of_probabilities_supports_online_application_over_unverified_telephone_claim; inadvertent_non_disclosure_of_prior_claims_entitles_insurer_to_void_if_insurer_demonstrates_it_would_not_have_offered_cover_at_all; renewal_documents_listing_disclosed_claims_constitute_evidence_of_claims_history_maintained_through_policy_renewals</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>DRN6785039.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="120" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>DRN7287812</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Not stated in document</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Motor insurance — Mr A's vehicle was stolen; RSA avoided the policy from inception for non-disclosure of an undisclosed 2008 theft claim (and a named driver's 2009 theft claim) and refused to meet the theft claim; RSA provided conflicting and inaccurate information throughout including conflicting accounts of how the claims were discovered and a letter from RSA's agent falsely stating Mr A had previously been found guilty of fraud; RSA's information failures caused Mr A to inadvertently remove the wrong claim from his CUE record and denied him the opportunity to seek alternative cover, leaving him uninsured when he had a separate accident in 2012</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft — vehicle stolen; specific circumstances of the theft not described; principal dispute concerns RSA's avoidance of the policy for non-disclosure and the consequential uninsured accident loss arising from RSA's handling failures</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Undisclosed 2008 theft claim (Mr A's own) and named driver's 2009 theft claim — RSA demonstrated it would not have offered cover had the 2008 theft claim been disclosed; policy avoided from inception; theft claim not paid</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Mr A: RSA provided conflicting information about how claims were discovered (claimed CUE was checked when evidence suggests it wasn't); RSA gave inaccurate claim dates that confused Mr A into inadvertently removing the real 2010 claim from his CUE record with the previous insurer; RSA falsely stated he had been found guilty of fraud causing business harm. RSA: Mr A failed to disclose 2008 theft claim in answer to a clear 5-year claims question; avoidance was correct; previous insurer confirmed two claims. FOS: non-disclosure of 2008 theft claim is undisputed — avoidance is reasonable and voidance may remain; however RSA created significant confusion through conflicting and inaccurate information; RSA could have avoided the policy in August 2011 when it had the information — Mr A could then have sought alternative cover and been insured at the time of his 2012 accident; RSA's inaccurate information caused Mr A to remove the wrong claim; false fraud allegation caused significant distress and inconvenience — £800 compensation appropriate</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>RSA to pay Mr A's 2012 accident damage claim with 8% simple interest from date of loss to date of settlement; RSA to pay £800 compensation for distress and inconvenience caused by poor customer service including false fraud allegation; voidance may remain on Mr A's record; no other award</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>An insurer that provides conflicting and inaccurate information about the basis for a non-disclosure avoidance may be required to pay claims it would otherwise be entitled to decline — where the insurer's own information failures prevented the policyholder from taking corrective action (seeking alternative cover) and the policyholder was consequently uninsured for a subsequent loss, the insurer bears responsibility for that loss; an insurer must not state in official correspondence that a policyholder has previously been found guilty of fraud when this is false — doing so causes significant reputational and business harm and warrants substantial D&amp;I compensation; while an insurer may legitimately avoid a policy for undisclosed theft claims, inaccurate information about how those claims were discovered can give rise to consequential liability if it prevents the policyholder from responding appropriately and seeking alternative cover</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>Recording of the pivotal August 2011 phone call between RSA and Mr A (not available to FOS); confirmed account from previous insurer of exactly what was communicated to RSA (disputed accounts between RSA and previous insurer)</t>
+        </is>
+      </c>
+      <c r="R38" s="3" t="inlineStr">
+        <is>
+          <t>Non-disclosure of 2008 theft claim undisputed — RSA entitled to avoid policy; but RSA provided conflicting and inaccurate information throughout (claimed CUE was checked but evidence strongly suggests it was not; gave inaccurate claim dates to Mr A); RSA's inaccurate information caused Mr A to contact previous insurer and inadvertently change the wrong claim record; RSA could have avoided the policy in August 2011 with the information it had — Mr A would then have been able to seek alternative cover and been insured for the 2012 accident; RSA should therefore pay for the accident damage; false fraud allegation caused significant distress and potential business harm — £800 compensation appropriate; voidance stands</t>
+        </is>
+      </c>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>When communicating with a policyholder about a non-disclosure avoidance, insurers must provide accurate and consistent information about how the undisclosed claims were discovered — conflicting accounts of the investigation undermine the avoidance process and may result in consequential liability for subsequent uninsured losses; a single false allegation of fraud in official correspondence can expose an insurer to substantial D&amp;I compensation even where the underlying avoidance decision is correct; insurers should act promptly once they identify non-disclosure — delay in avoiding a policy can extend the period during which the policyholder remains uninsured and unable to seek alternative cover</t>
+        </is>
+      </c>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_provides_conflicting_inaccurate_information_about_non_disclosure_investigation AND policyholder_cannot_seek_alternative_cover_as_a_result THEN insurer_may_be_liable_for_subsequent_uninsured_losses; IF insurer_sends_official_correspondence_falsely_alleging_prior_fraud_conviction THEN substantial_DI_compensation_warranted_regardless_of_underlying_avoidance_correctness; insurer_must_provide_accurate_consistent_account_of_how_undisclosed_claims_were_discovered; IF insurer_could_have_avoided_policy_earlier_with_correct_information_and_did_not THEN insurer_bears_responsibility_for_losses_that_occurred_in_gap_during_which_policyholder_was_uninsured</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>DRN7287812.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="120" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>THEFT-038</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>DRN8409372</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Zurich Insurance PLC</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>9 Jan 2017</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Home contents insurance — Mr and Mrs G complained that Zurich unfairly applied an increased compulsory excess (a special endorsement of £500 for any future jewellery loss) at their 2015 renewal in response to their recent claims history including theft claims; the endorsement required disclosure to prospective insurers and they said it prevented them obtaining competitive renewal quotes elsewhere</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Jewellery theft from home — the underlying theft claims (previous incidents recorded by Zurich) involved the theft of jewellery from the home; specific method not described; this case concerns the consequence of those recorded claims on renewal terms, not the circumstances of the theft itself</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — no current theft claim declined; dispute concerns Zurich's decision to apply a compulsory £500 jewellery excess endorsement at renewal based on Mr and Mrs G's recent claims history (including theft claims)</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>Mr and Mrs G: only one theft claim was made not two (addressed in a separate FOS complaint reference); if only one claim recorded, only one special term should have been applied; Zurich should remove the increased excess both historically and for the future. Zurich: three or more claims triggers referral to underwriters; renewal terms are offered at underwriters' discretion; increased excess fairly applied in line with internal guidelines; almost two months' notice given. FOS: Zurich's underwriting criteria show policyholders with three or more claims are referred to underwriters and renewal terms are at underwriters' discretion; Zurich demonstrated the endorsement was applied consistently with its internal guidelines; annual contract — no obligation to renew on the same terms as previous years; two months' notice to broker is reasonable; endorsement requiring disclosure to prospective insurers is how insurance works — some insurers declining to offer cover because of the endorsed excess does not make the endorsement unfair; question of whether one or two theft claims were correctly recorded is being addressed under a separate FOS complaint reference; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Zurich fairly applied an increased jewellery excess endorsement at renewal in line with its underwriting criteria and internal guidelines; annual contracts can be renewed on different terms; two months' notice was reasonable; the endorsement's required disclosure to prospective insurers is a standard insurance consequence, not an unfair practice in itself</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P39" s="5" t="inlineStr">
+        <is>
+          <t>An insurer is entitled to apply a special excess endorsement or increase the policy excess at renewal based on the policyholder's claims history — there is no obligation to renew an annual home insurance contract on the same terms as previous years; a special endorsement applied at renewal must be disclosed to prospective insurers when the policyholder seeks alternative quotes — the fact that disclosure makes other insurers less willing to offer competitive cover does not make the original endorsement unfair; where an insurer's internal underwriting criteria require referral to underwriters for policyholders with three or more claims and renewal terms are at underwriters' discretion, an endorsement applied consistently with those criteria is a reasonable exercise of underwriting judgment; a dispute about whether the number of underlying claims was correctly recorded is a separate complaint that must be brought independently</t>
+        </is>
+      </c>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Resolution of the parallel complaint about whether one or two theft claims were correctly recorded — FOS accepted Zurich's claim count of two for the purposes of this renewal terms complaint pending outcome of the separate FOS reference</t>
+        </is>
+      </c>
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>Zurich's evidence shows three or more claims triggers underwriter referral and renewal terms offered at underwriter discretion; increased jewellery excess endorsed to policy consistently with internal guidelines; annual contract — no renewal on same terms obligation; almost two months' notice given to broker before renewal (reasonable); endorsement requires disclosure to prospective insurers — standard insurance practice; some prospective insurers declining due to disclosed endorsement does not make the endorsement unfair; complaint about claim count being looked at under a separate reference; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S39" s="5" t="inlineStr">
+        <is>
+          <t>When applying special excess endorsements at renewal based on claims history, insurers must document that they have followed their own underwriting criteria for referral and endorsement application — consistent application of internal guidelines is the primary defence to a challenge that the endorsement is unfair; handlers should advise policyholders at renewal that any special endorsements must be disclosed to prospective insurers when seeking alternative quotes, managing expectations about market availability</t>
+        </is>
+      </c>
+      <c r="T39" s="5" t="inlineStr">
+        <is>
+          <t>IF claims_history_triggers_insurer_referral_to_underwriters_per_internal_criteria AND underwriter_applies_increased_excess_endorsement THEN renewal_endorsement_is_fair_exercise_of_underwriting_discretion; special_excess_endorsement_must_be_disclosed_to_prospective_insurers_when_seeking_alternative_quotes; fact_that_prospective_insurers_decline_due_to_disclosed_endorsement_does_not_make_the_endorsement_unfair; dispute_about_number_of_underlying_theft_claims_correctly_recorded_must_be_brought_as_separate_complaint</t>
+        </is>
+      </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>DRN8409372.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="120" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>THEFT-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>DRN8838516</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Saga Services Limited</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>16 Apr 2018</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Motor (car) insurance — Mr W's car insurance premium increased by approximately 20% at renewal; a further increase was applied when Mr W disclosed the theft of a motorcycle insured under a separate motor policy; Mr W complained that a motorcycle theft claim on a different policy should not affect his car insurance premium</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Motor vehicle theft (motorcycle) on a separate motor policy — motorcycle stolen and claimed under a different motor insurance policy; specific circumstances of theft not described; the motorcycle theft claim was disclosed at car insurance renewal and factored into the car insurance pricing by Saga's underwriters</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Motor vehicle (personal car insurance)</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — no claim declined; dispute concerns Saga's decision to increase car insurance renewal premium following disclosure of a motorcycle theft claim on a separate motor policy</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Mr W: unfair that a motorcycle theft claim on a separate policy affects his car insurance premium; pricing criteria must be underhand if they cannot be disclosed; surcharge is not morally fair. Saga: motorcycle theft is a motor claim that underwriters factor into any motor insurance pricing; pricing criteria are commercially sensitive but applied consistently to all policyholders in comparable circumstances; £37 loyalty discount offered. FOS: Saga's pricing information was reviewed and found to be applied consistently to all policyholders in comparable circumstances; motorcycle theft is a motor claim relevant to all motor insurance (both motorcycles and cars are motor vehicles requiring insurance for legal road use); pricing algorithms and criteria are legitimately commercially sensitive — insurers are not required to disclose them to policyholders; no unfair treatment of Mr W</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Saga fairly increased car insurance renewal premium to reflect the motorcycle theft claim on a separate motor policy; insurers are entitled to consider any motor claim (including claims on other motor policies) when pricing motor insurance; commercially sensitive pricing criteria do not need to be disclosed to policyholders</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr">
+        <is>
+          <t>An insurer may legitimately factor in claims made under separate motor insurance policies when pricing a motor insurance renewal — motorcycles and cars are both motor vehicles requiring insurance for legal road use and claims on either are relevant risk factors; commercially sensitive pricing algorithms and criteria do not need to be disclosed to policyholders — the insurer need only demonstrate to FOS that the pricing is applied consistently to all comparable policyholders; a motorcycle theft claim on a separate policy is correctly classified as a fault/bonus-disallowed claim where the insurer cannot recover the claim payment from a third party, and it is not unreasonable for a subsequent insurer to factor this into motor insurance pricing</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>No material missing evidence — Saga's pricing criteria were reviewed by FOS (as commercially sensitive information) and found to be consistently applied to all comparable policyholders</t>
+        </is>
+      </c>
+      <c r="R40" s="3" t="inlineStr">
+        <is>
+          <t>Saga demonstrated its pricing was applied consistently to all comparable policyholders; motorcycle theft is a motor claim relevant to car insurance pricing — both are motor vehicles requiring legal insurance; pricing information is legitimately commercially sensitive and does not need to be disclosed to Mr W; £37 loyalty discount was offered; renewal price was given in advance and then updated when Mr W disclosed the motorcycle theft; no unfair treatment; complaint not upheld</t>
+        </is>
+      </c>
+      <c r="S40" s="3" t="inlineStr">
+        <is>
+          <t>Motor insurers may lawfully factor claims on any motor vehicle (including motorcycles or vehicles insured under different policies) into renewal pricing for car insurance — both are motor vehicles requiring legal road insurance; when a policyholder challenges a premium increase based on a claim on a separate motor policy, the insurer should demonstrate that its pricing criteria are consistently applied to comparable policyholders using commercially sensitive information reviewed by FOS if necessary</t>
+        </is>
+      </c>
+      <c r="T40" s="3" t="inlineStr">
+        <is>
+          <t>IF motorcycle_theft_claim_exists_on_separate_motor_policy AND car_insurance_is_being_renewed THEN motorcycle_theft_claim_is_a_relevant_motor_risk_factor_that_can_be_factored_into_car_insurance_premium; commercially_sensitive_pricing_criteria_need_not_be_disclosed_to_policyholders_if_demonstrated_to_be_consistently_applied; theft_claim_on_any_motor_vehicle_where_insurer_cannot_recover_costs_is_fault_bonus_disallowed_claim_relevant_to_all_future_motor_insurance_pricing</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>DRN8838516.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>